<commit_message>
Rerun the pre-crisis check on the corrected data (seed 13)
Same fixes as the seed 42 worktree: credit_gap_missing dropped at load in rt2b,
nfa_g replaced by nfa_gdp, 'crisis' excluded from micro_cols, threshold metrics
left empty (one test year has no evaluated predecessor), and the A46
falsification baseline added. rt2a/rt2b returned to tools/run_pipeline.py.

The falsification rule scores AUROC 1.000 here too.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/results/12a_gran/results_12a_isolate_gran_final.xlsx
+++ b/outputs/results/12a_gran/results_12a_isolate_gran_final.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:W31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,65 +462,75 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>threshold_from_year</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>test_optimal_threshold</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>tp</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>fp</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>fn</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>tn</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>f1</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>precision</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>miss_rate</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>false_alarm_rate</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>accuracy</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>loss_07</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>loss_08</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>loss_09</t>
         </is>
@@ -555,46 +565,52 @@
         <v>0.3302682062847694</v>
       </c>
       <c r="H2" t="n">
+        <v>0.4134512387890711</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J2" t="n">
         <v>0.01663706238879454</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L2" t="n">
         <v>10</v>
       </c>
-      <c r="J2" t="n">
-        <v>15</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
       <c r="M2" t="n">
-        <v>0.5714285714285714</v>
+        <v>4</v>
       </c>
       <c r="N2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O2" t="n">
-        <v>0.4</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>0.375</v>
       </c>
       <c r="R2" t="n">
         <v>0.4</v>
       </c>
       <c r="S2" t="n">
-        <v>0.3</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="T2" t="n">
-        <v>0.2</v>
+        <v>0.44</v>
       </c>
       <c r="U2" t="n">
-        <v>0.1</v>
+        <v>0.48</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.4533333333333334</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.4266666666666667</v>
       </c>
     </row>
     <row r="3">
@@ -617,55 +633,61 @@
         <v>2010</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5166666666666667</v>
+        <v>0.4266666666666667</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4386503256468932</v>
+        <v>0.3775350047792503</v>
       </c>
       <c r="G3" t="n">
-        <v>0.247256</v>
+        <v>0.2637679999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>0.32</v>
+        <v>0.05</v>
       </c>
       <c r="I3" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="K3" t="n">
         <v>10</v>
       </c>
-      <c r="J3" t="n">
-        <v>13</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
       <c r="L3" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6060606060606061</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" t="n">
-        <v>0.4347826086956522</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
       <c r="Q3" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.4</v>
       </c>
       <c r="R3" t="n">
-        <v>0.48</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0.26</v>
+        <v>1</v>
       </c>
       <c r="T3" t="n">
-        <v>0.1733333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="U3" t="n">
-        <v>0.08666666666666667</v>
+        <v>0.3</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="4">
@@ -697,46 +719,52 @@
         <v>0.3515652120113373</v>
       </c>
       <c r="H4" t="n">
+        <v>0.01242134533822536</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J4" t="n">
         <v>0.3752442896366119</v>
       </c>
-      <c r="I4" t="n">
+      <c r="K4" t="n">
         <v>10</v>
       </c>
-      <c r="J4" t="n">
-        <v>12</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
       <c r="L4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="M4" t="n">
-        <v>0.625</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="n">
-        <v>0.4545454545454545</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
       <c r="Q4" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="R4" t="n">
-        <v>0.52</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>0.24</v>
+        <v>1</v>
       </c>
       <c r="T4" t="n">
-        <v>0.16</v>
+        <v>0.4</v>
       </c>
       <c r="U4" t="n">
-        <v>0.08000000000000002</v>
+        <v>0.3</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="5">
@@ -759,55 +787,61 @@
         <v>2010</v>
       </c>
       <c r="E5" t="n">
-        <v>0.44</v>
+        <v>0.3733333333333333</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3808868908868909</v>
+        <v>0.3447409353931093</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4000947300528722</v>
+        <v>0.4266780619907374</v>
       </c>
       <c r="H5" t="n">
-        <v>0.03566289372715235</v>
+        <v>0.3394000401354165</v>
       </c>
       <c r="I5" t="n">
-        <v>10</v>
+        <v>2009</v>
       </c>
       <c r="J5" t="n">
-        <v>14</v>
+        <v>0.01051689927472469</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5882352941176471</v>
+        <v>7</v>
       </c>
       <c r="N5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O5" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="R5" t="n">
-        <v>0.44</v>
+        <v>0.7</v>
       </c>
       <c r="S5" t="n">
-        <v>0.28</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="T5" t="n">
-        <v>0.1866666666666667</v>
+        <v>0.4</v>
       </c>
       <c r="U5" t="n">
-        <v>0.09333333333333334</v>
+        <v>0.6499999999999999</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.6833333333333333</v>
       </c>
     </row>
     <row r="6">
@@ -830,55 +864,61 @@
         <v>2010</v>
       </c>
       <c r="E6" t="n">
-        <v>0.45</v>
+        <v>0.42</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3988636363636364</v>
+        <v>0.3954545454545455</v>
       </c>
       <c r="G6" t="n">
-        <v>0.379083972587156</v>
+        <v>0.3825089562866688</v>
       </c>
       <c r="H6" t="n">
-        <v>0.420814479638009</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.4208144796380091</v>
+      </c>
+      <c r="K6" t="n">
         <v>10</v>
       </c>
-      <c r="J6" t="n">
-        <v>14</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
       <c r="L6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P6" t="n">
         <v>1</v>
       </c>
-      <c r="M6" t="n">
-        <v>0.5882352941176471</v>
-      </c>
-      <c r="N6" t="n">
+      <c r="Q6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
         <v>1</v>
       </c>
-      <c r="O6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.9333333333333333</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.28</v>
-      </c>
       <c r="T6" t="n">
-        <v>0.1866666666666667</v>
+        <v>0.4</v>
       </c>
       <c r="U6" t="n">
-        <v>0.09333333333333334</v>
+        <v>0.3</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="7">
@@ -910,45 +950,51 @@
         <v>0.3083624220446608</v>
       </c>
       <c r="H7" t="n">
+        <v>0.04470937183400933</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J7" t="n">
         <v>0.1188634608818508</v>
       </c>
-      <c r="I7" t="n">
+      <c r="K7" t="n">
         <v>10</v>
       </c>
-      <c r="J7" t="n">
+      <c r="L7" t="n">
         <v>12</v>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
         <v>3</v>
       </c>
-      <c r="M7" t="n">
+      <c r="O7" t="n">
         <v>0.625</v>
       </c>
-      <c r="N7" t="n">
+      <c r="P7" t="n">
         <v>1</v>
       </c>
-      <c r="O7" t="n">
+      <c r="Q7" t="n">
         <v>0.4545454545454545</v>
       </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
         <v>0.8</v>
       </c>
-      <c r="R7" t="n">
+      <c r="T7" t="n">
         <v>0.52</v>
       </c>
-      <c r="S7" t="n">
+      <c r="U7" t="n">
         <v>0.24</v>
       </c>
-      <c r="T7" t="n">
+      <c r="V7" t="n">
         <v>0.16</v>
       </c>
-      <c r="U7" t="n">
+      <c r="W7" t="n">
         <v>0.08000000000000002</v>
       </c>
     </row>
@@ -978,49 +1024,55 @@
         <v>0.6510926399545325</v>
       </c>
       <c r="G8" t="n">
-        <v>0.24142315899945</v>
+        <v>0.2411413218184643</v>
       </c>
       <c r="H8" t="n">
-        <v>0.479564160817484</v>
+        <v>0.01663706238879454</v>
       </c>
       <c r="I8" t="n">
-        <v>9</v>
+        <v>2010</v>
       </c>
       <c r="J8" t="n">
-        <v>9</v>
+        <v>0.4787910456219109</v>
       </c>
       <c r="K8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" t="n">
+        <v>15</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P8" t="n">
         <v>1</v>
       </c>
-      <c r="L8" t="n">
-        <v>6</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.6428571428571429</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W8" t="n">
         <v>0.1</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="U8" t="n">
-        <v>0.15</v>
       </c>
     </row>
     <row r="9">
@@ -1043,55 +1095,61 @@
         <v>2011</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6533333333333333</v>
+        <v>0.6733333333333333</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5856434793276898</v>
+        <v>0.6154520917678812</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2230026896503645</v>
+        <v>0.2211137273991924</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3845475210954841</v>
+        <v>0.23</v>
       </c>
       <c r="I9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.388030396912549</v>
+      </c>
+      <c r="K9" t="n">
         <v>10</v>
       </c>
-      <c r="J9" t="n">
-        <v>10</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
       <c r="L9" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="M9" t="n">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
         <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>0.5</v>
+        <v>0.5882352941176471</v>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="R9" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0.2</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="T9" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.44</v>
       </c>
       <c r="U9" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.28</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.1866666666666667</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.09333333333333334</v>
       </c>
     </row>
     <row r="10">
@@ -1114,55 +1172,61 @@
         <v>2011</v>
       </c>
       <c r="E10" t="n">
-        <v>0.7533333333333334</v>
+        <v>0.7333333333333334</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6665909090909091</v>
+        <v>0.6168452380952381</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2561646401882172</v>
+        <v>0.2715207934379578</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1051026284694672</v>
+        <v>0.3752442896366119</v>
       </c>
       <c r="I10" t="n">
-        <v>8</v>
+        <v>2010</v>
       </c>
       <c r="J10" t="n">
+        <v>0.08176444470882416</v>
+      </c>
+      <c r="K10" t="n">
         <v>4</v>
       </c>
-      <c r="K10" t="n">
-        <v>2</v>
-      </c>
       <c r="L10" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
-        <v>0.7272727272727273</v>
+        <v>6</v>
       </c>
       <c r="N10" t="n">
-        <v>0.8</v>
+        <v>12</v>
       </c>
       <c r="O10" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4705882352941176</v>
       </c>
       <c r="P10" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="S10" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q10" t="n">
-        <v>0.2666666666666667</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0.22</v>
-      </c>
       <c r="T10" t="n">
-        <v>0.2133333333333334</v>
+        <v>0.64</v>
       </c>
       <c r="U10" t="n">
-        <v>0.2066666666666667</v>
+        <v>0.48</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -1185,55 +1249,61 @@
         <v>2011</v>
       </c>
       <c r="E11" t="n">
-        <v>0.7</v>
+        <v>0.6533333333333334</v>
       </c>
       <c r="F11" t="n">
-        <v>0.6983467023172906</v>
+        <v>0.6157869907869907</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2332489029133263</v>
+        <v>0.2217233377856964</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4910117331747179</v>
+        <v>0.01051689927472469</v>
       </c>
       <c r="I11" t="n">
-        <v>7</v>
+        <v>2010</v>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>0.4526163636573869</v>
       </c>
       <c r="K11" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="M11" t="n">
-        <v>0.6363636363636364</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="P11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U11" t="n">
         <v>0.3</v>
       </c>
-      <c r="Q11" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="T11" t="n">
-        <v>0.3066666666666666</v>
-      </c>
-      <c r="U11" t="n">
-        <v>0.3033333333333333</v>
+      <c r="V11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="12">
@@ -1256,55 +1326,61 @@
         <v>2011</v>
       </c>
       <c r="E12" t="n">
-        <v>0.5366666666666666</v>
+        <v>0.5166666666666667</v>
       </c>
       <c r="F12" t="n">
-        <v>0.4340909090909091</v>
+        <v>0.4133333333333333</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2656166240652603</v>
+        <v>0.3690381431586418</v>
       </c>
       <c r="H12" t="n">
-        <v>0.3287671232876714</v>
+        <v>0.4208144796380091</v>
       </c>
       <c r="I12" t="n">
-        <v>10</v>
+        <v>2010</v>
       </c>
       <c r="J12" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M12" t="n">
-        <v>0.625</v>
+        <v>7</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="O12" t="n">
-        <v>0.4545454545454545</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.8</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="R12" t="n">
-        <v>0.52</v>
+        <v>0.7</v>
       </c>
       <c r="S12" t="n">
-        <v>0.24</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="T12" t="n">
-        <v>0.16</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="U12" t="n">
-        <v>0.08000000000000002</v>
+        <v>0.57</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.6133333333333333</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.6566666666666666</v>
       </c>
     </row>
     <row r="13">
@@ -1327,55 +1403,61 @@
         <v>2011</v>
       </c>
       <c r="E13" t="n">
-        <v>0.88</v>
+        <v>0.7933333333333334</v>
       </c>
       <c r="F13" t="n">
-        <v>0.8263383838383839</v>
+        <v>0.65250999000999</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2879982548758644</v>
+        <v>0.243084979730181</v>
       </c>
       <c r="H13" t="n">
-        <v>0.005595969106936115</v>
+        <v>0.1188634608818508</v>
       </c>
       <c r="I13" t="n">
-        <v>9</v>
+        <v>2010</v>
       </c>
       <c r="J13" t="n">
+        <v>0.06268846301026465</v>
+      </c>
+      <c r="K13" t="n">
+        <v>7</v>
+      </c>
+      <c r="L13" t="n">
+        <v>4</v>
+      </c>
+      <c r="M13" t="n">
         <v>3</v>
       </c>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13" t="n">
-        <v>12</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.8181818181818182</v>
-      </c>
       <c r="N13" t="n">
-        <v>0.9</v>
+        <v>11</v>
       </c>
       <c r="O13" t="n">
-        <v>0.75</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="P13" t="n">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.2</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="R13" t="n">
-        <v>0.84</v>
+        <v>0.3</v>
       </c>
       <c r="S13" t="n">
-        <v>0.13</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="T13" t="n">
-        <v>0.12</v>
+        <v>0.72</v>
       </c>
       <c r="U13" t="n">
-        <v>0.11</v>
+        <v>0.29</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.2933333333333333</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.2966666666666667</v>
       </c>
     </row>
     <row r="14">
@@ -1404,49 +1486,55 @@
         <v>0.7106672494172493</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2015931568180839</v>
+        <v>0.2018707410647163</v>
       </c>
       <c r="H14" t="n">
-        <v>0.4839371869283402</v>
+        <v>0.4787910456219109</v>
       </c>
       <c r="I14" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.4835679444768404</v>
+      </c>
+      <c r="K14" t="n">
         <v>8</v>
       </c>
-      <c r="J14" t="n">
-        <v>5</v>
-      </c>
-      <c r="K14" t="n">
+      <c r="L14" t="n">
+        <v>7</v>
+      </c>
+      <c r="M14" t="n">
         <v>2</v>
       </c>
-      <c r="L14" t="n">
-        <v>10</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0.6956521739130435</v>
-      </c>
       <c r="N14" t="n">
+        <v>8</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="P14" t="n">
         <v>0.8</v>
       </c>
-      <c r="O14" t="n">
-        <v>0.6153846153846154</v>
-      </c>
-      <c r="P14" t="n">
+      <c r="Q14" t="n">
+        <v>0.5333333333333333</v>
+      </c>
+      <c r="R14" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q14" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0.72</v>
-      </c>
       <c r="S14" t="n">
-        <v>0.24</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="T14" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0.2533333333333334</v>
+      </c>
+      <c r="W14" t="n">
         <v>0.2266666666666667</v>
-      </c>
-      <c r="U14" t="n">
-        <v>0.2133333333333333</v>
       </c>
     </row>
     <row r="15">
@@ -1469,55 +1557,61 @@
         <v>2012</v>
       </c>
       <c r="E15" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.8894491129785247</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.171196325072302</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.388030396912549</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.5746658796136312</v>
+      </c>
+      <c r="K15" t="n">
+        <v>9</v>
+      </c>
+      <c r="L15" t="n">
+        <v>9</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="n">
+        <v>6</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="P15" t="n">
         <v>0.9</v>
       </c>
-      <c r="F15" t="n">
-        <v>0.9126315789473685</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.1729535948149485</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.6117757361783286</v>
-      </c>
-      <c r="I15" t="n">
-        <v>8</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>2</v>
-      </c>
-      <c r="L15" t="n">
-        <v>15</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O15" t="n">
-        <v>1</v>
-      </c>
-      <c r="P15" t="n">
+      <c r="Q15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="V15" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="S15" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="T15" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U15" t="n">
-        <v>0.18</v>
+      <c r="W15" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="16">
@@ -1540,55 +1634,61 @@
         <v>2012</v>
       </c>
       <c r="E16" t="n">
-        <v>0.8733333333333334</v>
+        <v>0.8333333333333333</v>
       </c>
       <c r="F16" t="n">
-        <v>0.8826388888888889</v>
+        <v>0.8421212121212119</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1501580774784088</v>
+        <v>0.1703834533691406</v>
       </c>
       <c r="H16" t="n">
-        <v>0.671759307384491</v>
+        <v>0.08176444470882416</v>
       </c>
       <c r="I16" t="n">
-        <v>8</v>
+        <v>2011</v>
       </c>
       <c r="J16" t="n">
+        <v>0.7821449637413025</v>
+      </c>
+      <c r="K16" t="n">
+        <v>10</v>
+      </c>
+      <c r="L16" t="n">
+        <v>12</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>3</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="P16" t="n">
         <v>1</v>
       </c>
-      <c r="K16" t="n">
-        <v>2</v>
-      </c>
-      <c r="L16" t="n">
-        <v>14</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0.8421052631578947</v>
-      </c>
-      <c r="N16" t="n">
+      <c r="Q16" t="n">
+        <v>0.4545454545454545</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
         <v>0.8</v>
       </c>
-      <c r="O16" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0.06666666666666667</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="S16" t="n">
+      <c r="T16" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="V16" t="n">
         <v>0.16</v>
       </c>
-      <c r="T16" t="n">
-        <v>0.1733333333333334</v>
-      </c>
-      <c r="U16" t="n">
-        <v>0.1866666666666667</v>
+      <c r="W16" t="n">
+        <v>0.08000000000000002</v>
       </c>
     </row>
     <row r="17">
@@ -1611,55 +1711,61 @@
         <v>2012</v>
       </c>
       <c r="E17" t="n">
-        <v>0.74</v>
+        <v>0.66</v>
       </c>
       <c r="F17" t="n">
-        <v>0.7488677988677989</v>
+        <v>0.7187579242223204</v>
       </c>
       <c r="G17" t="n">
-        <v>0.217466614056738</v>
+        <v>0.2278677573667343</v>
       </c>
       <c r="H17" t="n">
-        <v>0.4996605725769222</v>
+        <v>0.4526163636573869</v>
       </c>
       <c r="I17" t="n">
-        <v>9</v>
+        <v>2011</v>
       </c>
       <c r="J17" t="n">
-        <v>6</v>
+        <v>0.6116516177496127</v>
       </c>
       <c r="K17" t="n">
+        <v>10</v>
+      </c>
+      <c r="L17" t="n">
+        <v>13</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>2</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.6060606060606061</v>
+      </c>
+      <c r="P17" t="n">
         <v>1</v>
       </c>
-      <c r="L17" t="n">
-        <v>9</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="N17" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="P17" t="n">
-        <v>0.1</v>
-      </c>
       <c r="Q17" t="n">
-        <v>0.4</v>
+        <v>0.4347826086956522</v>
       </c>
       <c r="R17" t="n">
-        <v>0.72</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>0.19</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="T17" t="n">
-        <v>0.16</v>
+        <v>0.48</v>
       </c>
       <c r="U17" t="n">
-        <v>0.13</v>
+        <v>0.26</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0.1733333333333333</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0.08666666666666667</v>
       </c>
     </row>
     <row r="18">
@@ -1691,46 +1797,52 @@
         <v>0.1841320532431732</v>
       </c>
       <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J18" t="n">
         <v>0.7374566109182709</v>
       </c>
-      <c r="I18" t="n">
-        <v>8</v>
-      </c>
-      <c r="J18" t="n">
-        <v>3</v>
-      </c>
       <c r="K18" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L18" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M18" t="n">
-        <v>0.7619047619047619</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="P18" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V18" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q18" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="R18" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="S18" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="T18" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="U18" t="n">
-        <v>0.2</v>
+      <c r="W18" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="19">
@@ -1753,55 +1865,61 @@
         <v>2012</v>
       </c>
       <c r="E19" t="n">
-        <v>0.9</v>
+        <v>0.8533333333333333</v>
       </c>
       <c r="F19" t="n">
-        <v>0.9003588516746411</v>
+        <v>0.8536019536019536</v>
       </c>
       <c r="G19" t="n">
-        <v>0.1384474904804223</v>
+        <v>0.1611596878164202</v>
       </c>
       <c r="H19" t="n">
-        <v>0.7285815117256835</v>
+        <v>0.06268846301026465</v>
       </c>
       <c r="I19" t="n">
-        <v>7</v>
+        <v>2011</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>0.4175046489981734</v>
       </c>
       <c r="K19" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L19" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M19" t="n">
-        <v>0.8235294117647058</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>0.7</v>
+        <v>2</v>
       </c>
       <c r="O19" t="n">
+        <v>0.6060606060606061</v>
+      </c>
+      <c r="P19" t="n">
         <v>1</v>
       </c>
-      <c r="P19" t="n">
-        <v>0.3</v>
-      </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>0.4347826086956522</v>
       </c>
       <c r="R19" t="n">
-        <v>0.88</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>0.21</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="T19" t="n">
-        <v>0.24</v>
+        <v>0.48</v>
       </c>
       <c r="U19" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0.1733333333333333</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.08666666666666667</v>
       </c>
     </row>
     <row r="20">
@@ -1832,48 +1950,24 @@
       <c r="G20" t="n">
         <v>0.2155429920581876</v>
       </c>
-      <c r="H20" t="n">
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="n">
         <v>0.214396107376168</v>
       </c>
-      <c r="I20" t="n">
-        <v>8</v>
-      </c>
-      <c r="J20" t="n">
-        <v>6</v>
-      </c>
-      <c r="K20" t="n">
-        <v>2</v>
-      </c>
-      <c r="L20" t="n">
-        <v>9</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="S20" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="T20" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="U20" t="n">
-        <v>0.22</v>
-      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1895,56 +1989,32 @@
         <v>2011</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6733333333333333</v>
+        <v>0.7133333333333334</v>
       </c>
       <c r="F21" t="n">
-        <v>0.6533760683760683</v>
+        <v>0.6660673966556319</v>
       </c>
       <c r="G21" t="n">
-        <v>0.3209719999999999</v>
-      </c>
-      <c r="H21" t="n">
+        <v>0.313324</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="n">
         <v>0.02</v>
       </c>
-      <c r="I21" t="n">
-        <v>8</v>
-      </c>
-      <c r="J21" t="n">
-        <v>8</v>
-      </c>
-      <c r="K21" t="n">
-        <v>2</v>
-      </c>
-      <c r="L21" t="n">
-        <v>7</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.6153846153846154</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0.5333333333333333</v>
-      </c>
-      <c r="R21" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="S21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T21" t="n">
-        <v>0.2666666666666667</v>
-      </c>
-      <c r="U21" t="n">
-        <v>0.2333333333333334</v>
-      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1974,48 +2044,24 @@
       <c r="G22" t="n">
         <v>0.312720388174057</v>
       </c>
-      <c r="H22" t="n">
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="n">
         <v>0.004134990740567446</v>
       </c>
-      <c r="I22" t="n">
-        <v>9</v>
-      </c>
-      <c r="J22" t="n">
-        <v>8</v>
-      </c>
-      <c r="K22" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" t="n">
-        <v>7</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0.5294117647058824</v>
-      </c>
-      <c r="P22" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>0.5333333333333333</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="S22" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="T22" t="n">
-        <v>0.1866666666666667</v>
-      </c>
-      <c r="U22" t="n">
-        <v>0.1433333333333333</v>
-      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2037,56 +2083,32 @@
         <v>2011</v>
       </c>
       <c r="E23" t="n">
-        <v>0.8133333333333334</v>
+        <v>0.8200000000000001</v>
       </c>
       <c r="F23" t="n">
-        <v>0.798799762329174</v>
+        <v>0.779298245614035</v>
       </c>
       <c r="G23" t="n">
-        <v>0.1911382389981019</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.1807592812230448</v>
-      </c>
-      <c r="I23" t="n">
-        <v>8</v>
-      </c>
+        <v>0.1820167877012062</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="n">
-        <v>4</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>11</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0.7272727272727273</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="P23" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>0.2666666666666667</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="S23" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="T23" t="n">
-        <v>0.2133333333333334</v>
-      </c>
-      <c r="U23" t="n">
-        <v>0.2066666666666667</v>
-      </c>
+        <v>0.2224123462181918</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2108,56 +2130,32 @@
         <v>2011</v>
       </c>
       <c r="E24" t="n">
-        <v>0.5733333333333333</v>
+        <v>0.5466666666666666</v>
       </c>
       <c r="F24" t="n">
         <v>0.52</v>
       </c>
       <c r="G24" t="n">
-        <v>0.3427203439871637</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>10</v>
-      </c>
+        <v>0.3640205631252207</v>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="n">
-        <v>15</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="N24" t="n">
-        <v>1</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1</v>
-      </c>
-      <c r="R24" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S24" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T24" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="U24" t="n">
-        <v>0.1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2187,48 +2185,24 @@
       <c r="G25" t="n">
         <v>0.2764459795613017</v>
       </c>
-      <c r="H25" t="n">
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="n">
         <v>0.003988136469010892</v>
       </c>
-      <c r="I25" t="n">
-        <v>8</v>
-      </c>
-      <c r="J25" t="n">
-        <v>1</v>
-      </c>
-      <c r="K25" t="n">
-        <v>2</v>
-      </c>
-      <c r="L25" t="n">
-        <v>14</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0.8421052631578947</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="P25" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>0.06666666666666667</v>
-      </c>
-      <c r="R25" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="S25" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="T25" t="n">
-        <v>0.1733333333333334</v>
-      </c>
-      <c r="U25" t="n">
-        <v>0.1866666666666667</v>
-      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2259,46 +2233,52 @@
         <v>0.1831261321893823</v>
       </c>
       <c r="H26" t="n">
+        <v>0.214396107376168</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J26" t="n">
         <v>0.1466912697483659</v>
       </c>
-      <c r="I26" t="n">
-        <v>10</v>
-      </c>
-      <c r="J26" t="n">
-        <v>7</v>
-      </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L26" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M26" t="n">
-        <v>0.7407407407407407</v>
+        <v>4</v>
       </c>
       <c r="N26" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="O26" t="n">
-        <v>0.5882352941176471</v>
+        <v>0.6</v>
       </c>
       <c r="P26" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.4666666666666667</v>
+        <v>0.6</v>
       </c>
       <c r="R26" t="n">
-        <v>0.72</v>
+        <v>0.4</v>
       </c>
       <c r="S26" t="n">
-        <v>0.14</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="T26" t="n">
-        <v>0.09333333333333334</v>
+        <v>0.68</v>
       </c>
       <c r="U26" t="n">
-        <v>0.04666666666666667</v>
+        <v>0.36</v>
+      </c>
+      <c r="V26" t="n">
+        <v>0.3733333333333334</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.3866666666666667</v>
       </c>
     </row>
     <row r="27">
@@ -2321,55 +2301,61 @@
         <v>2012</v>
       </c>
       <c r="E27" t="n">
-        <v>0.8866666666666666</v>
+        <v>0.88</v>
       </c>
       <c r="F27" t="n">
-        <v>0.8323841354723708</v>
+        <v>0.8591117216117214</v>
       </c>
       <c r="G27" t="n">
-        <v>0.216776</v>
+        <v>0.214724</v>
       </c>
       <c r="H27" t="n">
-        <v>0.25</v>
+        <v>0.02</v>
       </c>
       <c r="I27" t="n">
-        <v>7</v>
+        <v>2011</v>
       </c>
       <c r="J27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K27" t="n">
+        <v>10</v>
+      </c>
+      <c r="L27" t="n">
+        <v>12</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>3</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="P27" t="n">
         <v>1</v>
       </c>
-      <c r="K27" t="n">
-        <v>3</v>
-      </c>
-      <c r="L27" t="n">
-        <v>14</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="O27" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="P27" t="n">
-        <v>0.3</v>
-      </c>
       <c r="Q27" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.4545454545454545</v>
       </c>
       <c r="R27" t="n">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>0.23</v>
+        <v>0.8</v>
       </c>
       <c r="T27" t="n">
-        <v>0.2533333333333333</v>
+        <v>0.52</v>
       </c>
       <c r="U27" t="n">
-        <v>0.2766666666666667</v>
+        <v>0.24</v>
+      </c>
+      <c r="V27" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.08000000000000002</v>
       </c>
     </row>
     <row r="28">
@@ -2401,46 +2387,52 @@
         <v>0.2171606421470642</v>
       </c>
       <c r="H28" t="n">
+        <v>0.004134990740567446</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J28" t="n">
         <v>0.03543443605303764</v>
       </c>
-      <c r="I28" t="n">
-        <v>8</v>
-      </c>
-      <c r="J28" t="n">
-        <v>3</v>
-      </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L28" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M28" t="n">
-        <v>0.7619047619047619</v>
+        <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>0.8</v>
+        <v>5</v>
       </c>
       <c r="O28" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.6206896551724138</v>
       </c>
       <c r="P28" t="n">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.2</v>
+        <v>0.4736842105263158</v>
       </c>
       <c r="R28" t="n">
-        <v>0.8</v>
+        <v>0.1</v>
       </c>
       <c r="S28" t="n">
-        <v>0.2</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="T28" t="n">
-        <v>0.2</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="U28" t="n">
-        <v>0.2</v>
+        <v>0.27</v>
+      </c>
+      <c r="V28" t="n">
+        <v>0.2133333333333333</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.1566666666666667</v>
       </c>
     </row>
     <row r="29">
@@ -2463,55 +2455,61 @@
         <v>2012</v>
       </c>
       <c r="E29" t="n">
-        <v>0.8266666666666667</v>
+        <v>0.8200000000000001</v>
       </c>
       <c r="F29" t="n">
-        <v>0.8286247086247086</v>
+        <v>0.7794839218752262</v>
       </c>
       <c r="G29" t="n">
-        <v>0.1741227916710872</v>
+        <v>0.1718519934284202</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1691485916788619</v>
+        <v>0.2224123462181918</v>
       </c>
       <c r="I29" t="n">
-        <v>9</v>
+        <v>2011</v>
       </c>
       <c r="J29" t="n">
-        <v>4</v>
+        <v>0.1946459690721781</v>
       </c>
       <c r="K29" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L29" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="M29" t="n">
-        <v>0.7826086956521739</v>
+        <v>2</v>
       </c>
       <c r="N29" t="n">
-        <v>0.9</v>
+        <v>12</v>
       </c>
       <c r="O29" t="n">
-        <v>0.6923076923076923</v>
+        <v>0.7619047619047619</v>
       </c>
       <c r="P29" t="n">
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="R29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="S29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="T29" t="n">
         <v>0.8</v>
       </c>
-      <c r="S29" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="T29" t="n">
-        <v>0.1333333333333334</v>
-      </c>
       <c r="U29" t="n">
-        <v>0.1166666666666667</v>
+        <v>0.2</v>
+      </c>
+      <c r="V29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W29" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="30">
@@ -2534,54 +2532,60 @@
         <v>2012</v>
       </c>
       <c r="E30" t="n">
-        <v>0.5666666666666667</v>
+        <v>0.54</v>
       </c>
       <c r="F30" t="n">
         <v>0.4533333333333334</v>
       </c>
       <c r="G30" t="n">
-        <v>0.3511584918577925</v>
+        <v>0.3770100873979694</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
       </c>
       <c r="I30" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
         <v>10</v>
       </c>
-      <c r="J30" t="n">
+      <c r="L30" t="n">
         <v>15</v>
       </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
       <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
         <v>0.5714285714285714</v>
       </c>
-      <c r="N30" t="n">
+      <c r="P30" t="n">
         <v>1</v>
       </c>
-      <c r="O30" t="n">
+      <c r="Q30" t="n">
         <v>0.4</v>
       </c>
-      <c r="P30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" t="n">
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="n">
         <v>1</v>
       </c>
-      <c r="R30" t="n">
+      <c r="T30" t="n">
         <v>0.4</v>
       </c>
-      <c r="S30" t="n">
+      <c r="U30" t="n">
         <v>0.3</v>
       </c>
-      <c r="T30" t="n">
+      <c r="V30" t="n">
         <v>0.2</v>
       </c>
-      <c r="U30" t="n">
+      <c r="W30" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -2614,46 +2618,52 @@
         <v>0.2019680095014026</v>
       </c>
       <c r="H31" t="n">
+        <v>0.003988136469010892</v>
+      </c>
+      <c r="I31" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J31" t="n">
         <v>0.02090703665427157</v>
       </c>
-      <c r="I31" t="n">
+      <c r="K31" t="n">
         <v>9</v>
       </c>
-      <c r="J31" t="n">
-        <v>2</v>
-      </c>
-      <c r="K31" t="n">
+      <c r="L31" t="n">
+        <v>7</v>
+      </c>
+      <c r="M31" t="n">
         <v>1</v>
       </c>
-      <c r="L31" t="n">
-        <v>13</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0.8571428571428571</v>
-      </c>
       <c r="N31" t="n">
+        <v>8</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0.6923076923076923</v>
+      </c>
+      <c r="P31" t="n">
         <v>0.9</v>
       </c>
-      <c r="O31" t="n">
-        <v>0.8181818181818182</v>
-      </c>
-      <c r="P31" t="n">
+      <c r="Q31" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="R31" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q31" t="n">
-        <v>0.1333333333333333</v>
-      </c>
-      <c r="R31" t="n">
-        <v>0.88</v>
-      </c>
       <c r="S31" t="n">
-        <v>0.11</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="T31" t="n">
-        <v>0.1066666666666667</v>
+        <v>0.68</v>
       </c>
       <c r="U31" t="n">
-        <v>0.1033333333333333</v>
+        <v>0.21</v>
+      </c>
+      <c r="V31" t="n">
+        <v>0.1733333333333333</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0.1366666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -2689,7 +2699,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.603</v>
+        <v>0.587</v>
       </c>
     </row>
     <row r="3">
@@ -2699,7 +2709,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.782</v>
+        <v>0.738</v>
       </c>
     </row>
     <row r="4">
@@ -2719,7 +2729,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.627</v>
+        <v>0.5620000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -2729,7 +2739,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.656</v>
       </c>
     </row>
     <row r="7">
@@ -2739,7 +2749,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.711</v>
+        <v>0.6909999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2815,25 +2825,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.603</v>
+        <v>0.587</v>
       </c>
       <c r="D2" t="n">
-        <v>0.658</v>
+        <v>0.499</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.767</v>
       </c>
       <c r="F2" t="n">
-        <v>0.533</v>
+        <v>0.41</v>
       </c>
       <c r="G2" t="n">
-        <v>0.067</v>
+        <v>0.233</v>
       </c>
       <c r="H2" t="n">
-        <v>0.644</v>
+        <v>0.756</v>
       </c>
       <c r="I2" t="n">
-        <v>0.182</v>
+        <v>0.338</v>
       </c>
     </row>
     <row r="3">
@@ -2848,25 +2858,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.782</v>
+        <v>0.738</v>
       </c>
       <c r="D3" t="n">
-        <v>0.756</v>
+        <v>0.633</v>
       </c>
       <c r="E3" t="n">
-        <v>0.867</v>
+        <v>0.9</v>
       </c>
       <c r="F3" t="n">
-        <v>0.735</v>
+        <v>0.509</v>
       </c>
       <c r="G3" t="n">
-        <v>0.133</v>
+        <v>0.1</v>
       </c>
       <c r="H3" t="n">
-        <v>0.333</v>
+        <v>0.644</v>
       </c>
       <c r="I3" t="n">
-        <v>0.173</v>
+        <v>0.209</v>
       </c>
     </row>
     <row r="4">
@@ -2884,22 +2894,22 @@
         <v>0.638</v>
       </c>
       <c r="D4" t="n">
-        <v>0.637</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="F4" t="n">
-        <v>0.505</v>
+        <v>0.436</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H4" t="n">
-        <v>0.644</v>
+        <v>0.711</v>
       </c>
       <c r="I4" t="n">
-        <v>0.209</v>
+        <v>0.302</v>
       </c>
     </row>
     <row r="5">
@@ -2914,25 +2924,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.627</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>0.648</v>
+        <v>0.488</v>
       </c>
       <c r="E5" t="n">
-        <v>0.867</v>
+        <v>0.767</v>
       </c>
       <c r="F5" t="n">
-        <v>0.533</v>
+        <v>0.369</v>
       </c>
       <c r="G5" t="n">
-        <v>0.133</v>
+        <v>0.233</v>
       </c>
       <c r="H5" t="n">
-        <v>0.556</v>
+        <v>0.8</v>
       </c>
       <c r="I5" t="n">
-        <v>0.218</v>
+        <v>0.347</v>
       </c>
     </row>
     <row r="6">
@@ -2947,25 +2957,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.656</v>
       </c>
       <c r="D6" t="n">
-        <v>0.721</v>
+        <v>0.601</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.967</v>
       </c>
       <c r="F6" t="n">
-        <v>0.645</v>
+        <v>0.439</v>
       </c>
       <c r="G6" t="n">
-        <v>0.067</v>
+        <v>0.033</v>
       </c>
       <c r="H6" t="n">
-        <v>0.511</v>
+        <v>0.844</v>
       </c>
       <c r="I6" t="n">
-        <v>0.156</v>
+        <v>0.196</v>
       </c>
     </row>
     <row r="7">
@@ -2980,25 +2990,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.711</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>0.731</v>
+        <v>0.556</v>
       </c>
       <c r="E7" t="n">
-        <v>0.867</v>
+        <v>0.8</v>
       </c>
       <c r="F7" t="n">
-        <v>0.67</v>
+        <v>0.475</v>
       </c>
       <c r="G7" t="n">
-        <v>0.133</v>
+        <v>0.2</v>
       </c>
       <c r="H7" t="n">
-        <v>0.378</v>
+        <v>0.667</v>
       </c>
       <c r="I7" t="n">
-        <v>0.182</v>
+        <v>0.293</v>
       </c>
     </row>
   </sheetData>
@@ -3044,7 +3054,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.603</v>
+        <v>0.587</v>
       </c>
     </row>
     <row r="3">
@@ -3054,7 +3064,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.782</v>
+        <v>0.738</v>
       </c>
     </row>
     <row r="4">
@@ -3074,7 +3084,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.627</v>
+        <v>0.5620000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -3084,7 +3094,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.656</v>
       </c>
     </row>
     <row r="7">
@@ -3094,7 +3104,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.711</v>
+        <v>0.6909999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -3109,7 +3119,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.57</v>
+        <v>0.543</v>
       </c>
     </row>
     <row r="9">
@@ -3149,7 +3159,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.78</v>
+        <v>0.797</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Rerun the pre-crisis check on the corrected data (seed 7)
Same fixes as the seed 42 worktree: credit_gap_missing dropped at load in rt2b,
nfa_g replaced by nfa_gdp, 'crisis' excluded from micro_cols, threshold metrics
left empty (one test year has no evaluated predecessor), and the A46
falsification baseline added. rt2a/rt2b returned to tools/run_pipeline.py.

The falsification rule scores AUROC 1.000 here too.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/results/12a_gran/results_12a_isolate_gran_final.xlsx
+++ b/outputs/results/12a_gran/results_12a_isolate_gran_final.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:W31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,65 +462,75 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>threshold_from_year</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>test_optimal_threshold</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>tp</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>fp</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>fn</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>tn</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>f1</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>precision</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>miss_rate</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>false_alarm_rate</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>accuracy</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>loss_07</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>loss_08</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>loss_09</t>
         </is>
@@ -555,46 +565,52 @@
         <v>0.3302682062847694</v>
       </c>
       <c r="H2" t="n">
+        <v>0.4134512387890711</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J2" t="n">
         <v>0.01663706238879454</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L2" t="n">
         <v>10</v>
       </c>
-      <c r="J2" t="n">
-        <v>15</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
       <c r="M2" t="n">
-        <v>0.5714285714285714</v>
+        <v>4</v>
       </c>
       <c r="N2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O2" t="n">
-        <v>0.4</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>0.375</v>
       </c>
       <c r="R2" t="n">
         <v>0.4</v>
       </c>
       <c r="S2" t="n">
-        <v>0.3</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="T2" t="n">
-        <v>0.2</v>
+        <v>0.44</v>
       </c>
       <c r="U2" t="n">
-        <v>0.1</v>
+        <v>0.48</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.4533333333333334</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.4266666666666667</v>
       </c>
     </row>
     <row r="3">
@@ -617,55 +633,61 @@
         <v>2010</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5166666666666667</v>
+        <v>0.4033333333333333</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4386503256468932</v>
+        <v>0.3503763885416867</v>
       </c>
       <c r="G3" t="n">
-        <v>0.247256</v>
+        <v>0.258248</v>
       </c>
       <c r="H3" t="n">
-        <v>0.32</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I3" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K3" t="n">
         <v>10</v>
       </c>
-      <c r="J3" t="n">
-        <v>13</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
       <c r="L3" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6060606060606061</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" t="n">
-        <v>0.4347826086956522</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
       <c r="Q3" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.4</v>
       </c>
       <c r="R3" t="n">
-        <v>0.48</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0.26</v>
+        <v>1</v>
       </c>
       <c r="T3" t="n">
-        <v>0.1733333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="U3" t="n">
-        <v>0.08666666666666667</v>
+        <v>0.3</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="4">
@@ -697,46 +719,52 @@
         <v>0.3515652120113373</v>
       </c>
       <c r="H4" t="n">
+        <v>0.01242134533822536</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J4" t="n">
         <v>0.3752442896366119</v>
       </c>
-      <c r="I4" t="n">
+      <c r="K4" t="n">
         <v>10</v>
       </c>
-      <c r="J4" t="n">
-        <v>12</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
       <c r="L4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="M4" t="n">
-        <v>0.625</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="n">
-        <v>0.4545454545454545</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
       <c r="Q4" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="R4" t="n">
-        <v>0.52</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>0.24</v>
+        <v>1</v>
       </c>
       <c r="T4" t="n">
-        <v>0.16</v>
+        <v>0.4</v>
       </c>
       <c r="U4" t="n">
-        <v>0.08000000000000002</v>
+        <v>0.3</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="5">
@@ -759,55 +787,61 @@
         <v>2010</v>
       </c>
       <c r="E5" t="n">
-        <v>0.44</v>
+        <v>0.4333333333333333</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3808868908868909</v>
+        <v>0.3794910545549932</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4000947300528722</v>
+        <v>0.4065702977579634</v>
       </c>
       <c r="H5" t="n">
-        <v>0.03566289372715235</v>
+        <v>0.2847703550402944</v>
       </c>
       <c r="I5" t="n">
-        <v>10</v>
+        <v>2009</v>
       </c>
       <c r="J5" t="n">
-        <v>14</v>
+        <v>0.008090484841300941</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5882352941176471</v>
+        <v>4</v>
       </c>
       <c r="N5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="O5" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="R5" t="n">
-        <v>0.44</v>
+        <v>0.4</v>
       </c>
       <c r="S5" t="n">
-        <v>0.28</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="T5" t="n">
-        <v>0.1866666666666667</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="U5" t="n">
-        <v>0.09333333333333334</v>
+        <v>0.4199999999999999</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.4133333333333334</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.4066666666666667</v>
       </c>
     </row>
     <row r="6">
@@ -830,55 +864,61 @@
         <v>2010</v>
       </c>
       <c r="E6" t="n">
-        <v>0.45</v>
+        <v>0.4266666666666666</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3988636363636364</v>
+        <v>0.3727272727272727</v>
       </c>
       <c r="G6" t="n">
-        <v>0.379083972587156</v>
+        <v>0.3876744526264135</v>
       </c>
       <c r="H6" t="n">
-        <v>0.420814479638009</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.4208144796380091</v>
+      </c>
+      <c r="K6" t="n">
         <v>10</v>
       </c>
-      <c r="J6" t="n">
-        <v>14</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
       <c r="L6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P6" t="n">
         <v>1</v>
       </c>
-      <c r="M6" t="n">
-        <v>0.5882352941176471</v>
-      </c>
-      <c r="N6" t="n">
+      <c r="Q6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
         <v>1</v>
       </c>
-      <c r="O6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.9333333333333333</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.28</v>
-      </c>
       <c r="T6" t="n">
-        <v>0.1866666666666667</v>
+        <v>0.4</v>
       </c>
       <c r="U6" t="n">
-        <v>0.09333333333333334</v>
+        <v>0.3</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="7">
@@ -910,45 +950,51 @@
         <v>0.3083624220446608</v>
       </c>
       <c r="H7" t="n">
+        <v>0.04470937183400933</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J7" t="n">
         <v>0.1188634608818508</v>
       </c>
-      <c r="I7" t="n">
+      <c r="K7" t="n">
         <v>10</v>
       </c>
-      <c r="J7" t="n">
+      <c r="L7" t="n">
         <v>12</v>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
         <v>3</v>
       </c>
-      <c r="M7" t="n">
+      <c r="O7" t="n">
         <v>0.625</v>
       </c>
-      <c r="N7" t="n">
+      <c r="P7" t="n">
         <v>1</v>
       </c>
-      <c r="O7" t="n">
+      <c r="Q7" t="n">
         <v>0.4545454545454545</v>
       </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
         <v>0.8</v>
       </c>
-      <c r="R7" t="n">
+      <c r="T7" t="n">
         <v>0.52</v>
       </c>
-      <c r="S7" t="n">
+      <c r="U7" t="n">
         <v>0.24</v>
       </c>
-      <c r="T7" t="n">
+      <c r="V7" t="n">
         <v>0.16</v>
       </c>
-      <c r="U7" t="n">
+      <c r="W7" t="n">
         <v>0.08000000000000002</v>
       </c>
     </row>
@@ -972,55 +1018,61 @@
         <v>2011</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.66</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6510926399545325</v>
+        <v>0.6472464861083786</v>
       </c>
       <c r="G8" t="n">
-        <v>0.24142315899945</v>
+        <v>0.2419525425996561</v>
       </c>
       <c r="H8" t="n">
-        <v>0.479564160817484</v>
+        <v>0.01663706238879454</v>
       </c>
       <c r="I8" t="n">
-        <v>9</v>
+        <v>2010</v>
       </c>
       <c r="J8" t="n">
-        <v>9</v>
+        <v>0.4809997972661145</v>
       </c>
       <c r="K8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" t="n">
+        <v>15</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P8" t="n">
         <v>1</v>
       </c>
-      <c r="L8" t="n">
-        <v>6</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.6428571428571429</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W8" t="n">
         <v>0.1</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="U8" t="n">
-        <v>0.15</v>
       </c>
     </row>
     <row r="9">
@@ -1043,55 +1095,61 @@
         <v>2011</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6533333333333333</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5856434793276898</v>
+        <v>0.5384649122807017</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2230026896503645</v>
+        <v>0.2206403624401537</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3845475210954841</v>
+        <v>0.27</v>
       </c>
       <c r="I9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.3692332047685616</v>
+      </c>
+      <c r="K9" t="n">
         <v>10</v>
       </c>
-      <c r="J9" t="n">
-        <v>10</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
       <c r="L9" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="M9" t="n">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
+        <v>2</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.6060606060606061</v>
+      </c>
+      <c r="P9" t="n">
         <v>1</v>
       </c>
-      <c r="O9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
       <c r="Q9" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4347826086956522</v>
       </c>
       <c r="R9" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0.2</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="T9" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.48</v>
       </c>
       <c r="U9" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.26</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.1733333333333333</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.08666666666666667</v>
       </c>
     </row>
     <row r="10">
@@ -1114,55 +1172,61 @@
         <v>2011</v>
       </c>
       <c r="E10" t="n">
-        <v>0.7533333333333334</v>
+        <v>0.8266666666666667</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6665909090909091</v>
+        <v>0.7721336996336996</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2561646401882172</v>
+        <v>0.2054422944784164</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1051026284694672</v>
+        <v>0.3752442896366119</v>
       </c>
       <c r="I10" t="n">
-        <v>8</v>
+        <v>2010</v>
       </c>
       <c r="J10" t="n">
-        <v>4</v>
+        <v>0.0711463987827301</v>
       </c>
       <c r="K10" t="n">
+        <v>5</v>
+      </c>
+      <c r="L10" t="n">
         <v>2</v>
       </c>
-      <c r="L10" t="n">
-        <v>11</v>
-      </c>
       <c r="M10" t="n">
-        <v>0.7272727272727273</v>
+        <v>5</v>
       </c>
       <c r="N10" t="n">
-        <v>0.8</v>
+        <v>13</v>
       </c>
       <c r="O10" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5882352941176471</v>
       </c>
       <c r="P10" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="R10" t="n">
-        <v>0.76</v>
+        <v>0.5</v>
       </c>
       <c r="S10" t="n">
-        <v>0.22</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="T10" t="n">
-        <v>0.2133333333333334</v>
+        <v>0.72</v>
       </c>
       <c r="U10" t="n">
-        <v>0.2066666666666667</v>
+        <v>0.39</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.4266666666666667</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.4633333333333333</v>
       </c>
     </row>
     <row r="11">
@@ -1185,55 +1249,61 @@
         <v>2011</v>
       </c>
       <c r="E11" t="n">
-        <v>0.7</v>
+        <v>0.78</v>
       </c>
       <c r="F11" t="n">
-        <v>0.6983467023172906</v>
+        <v>0.7777686436893598</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2332489029133263</v>
+        <v>0.1979175996337955</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4910117331747179</v>
+        <v>0.008090484841300941</v>
       </c>
       <c r="I11" t="n">
-        <v>7</v>
+        <v>2010</v>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>0.5022939176665918</v>
       </c>
       <c r="K11" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="M11" t="n">
-        <v>0.6363636363636364</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="P11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U11" t="n">
         <v>0.3</v>
       </c>
-      <c r="Q11" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="T11" t="n">
-        <v>0.3066666666666666</v>
-      </c>
-      <c r="U11" t="n">
-        <v>0.3033333333333333</v>
+      <c r="V11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="12">
@@ -1256,55 +1326,61 @@
         <v>2011</v>
       </c>
       <c r="E12" t="n">
-        <v>0.5366666666666666</v>
+        <v>0.5166666666666667</v>
       </c>
       <c r="F12" t="n">
-        <v>0.4340909090909091</v>
+        <v>0.4133333333333333</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2656166240652603</v>
+        <v>0.3690381431586418</v>
       </c>
       <c r="H12" t="n">
-        <v>0.3287671232876714</v>
+        <v>0.4208144796380091</v>
       </c>
       <c r="I12" t="n">
-        <v>10</v>
+        <v>2010</v>
       </c>
       <c r="J12" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M12" t="n">
-        <v>0.625</v>
+        <v>7</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="O12" t="n">
-        <v>0.4545454545454545</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.8</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="R12" t="n">
-        <v>0.52</v>
+        <v>0.7</v>
       </c>
       <c r="S12" t="n">
-        <v>0.24</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="T12" t="n">
-        <v>0.16</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="U12" t="n">
-        <v>0.08000000000000002</v>
+        <v>0.57</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.6133333333333333</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.6566666666666666</v>
       </c>
     </row>
     <row r="13">
@@ -1327,55 +1403,61 @@
         <v>2011</v>
       </c>
       <c r="E13" t="n">
-        <v>0.88</v>
+        <v>0.8</v>
       </c>
       <c r="F13" t="n">
-        <v>0.8263383838383839</v>
+        <v>0.6808891108891107</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2879982548758644</v>
+        <v>0.2136637124822977</v>
       </c>
       <c r="H13" t="n">
-        <v>0.005595969106936115</v>
+        <v>0.1188634608818508</v>
       </c>
       <c r="I13" t="n">
-        <v>9</v>
+        <v>2010</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>0.1237974127607304</v>
       </c>
       <c r="K13" t="n">
+        <v>10</v>
+      </c>
+      <c r="L13" t="n">
+        <v>5</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
+        <v>10</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="P13" t="n">
         <v>1</v>
       </c>
-      <c r="L13" t="n">
-        <v>12</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.8181818181818182</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0.1</v>
-      </c>
       <c r="Q13" t="n">
-        <v>0.2</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="R13" t="n">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>0.13</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="T13" t="n">
-        <v>0.12</v>
+        <v>0.8</v>
       </c>
       <c r="U13" t="n">
-        <v>0.11</v>
+        <v>0.09999999999999999</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.06666666666666667</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="14">
@@ -1404,49 +1486,55 @@
         <v>0.7106672494172493</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2015931568180839</v>
+        <v>0.2017049809104933</v>
       </c>
       <c r="H14" t="n">
-        <v>0.4839371869283402</v>
+        <v>0.4809997972661145</v>
       </c>
       <c r="I14" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.4837862876896714</v>
+      </c>
+      <c r="K14" t="n">
         <v>8</v>
       </c>
-      <c r="J14" t="n">
-        <v>5</v>
-      </c>
-      <c r="K14" t="n">
+      <c r="L14" t="n">
+        <v>6</v>
+      </c>
+      <c r="M14" t="n">
         <v>2</v>
       </c>
-      <c r="L14" t="n">
-        <v>10</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0.6956521739130435</v>
-      </c>
       <c r="N14" t="n">
+        <v>9</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="P14" t="n">
         <v>0.8</v>
       </c>
-      <c r="O14" t="n">
-        <v>0.6153846153846154</v>
-      </c>
-      <c r="P14" t="n">
+      <c r="Q14" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="R14" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q14" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0.72</v>
-      </c>
       <c r="S14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="V14" t="n">
         <v>0.24</v>
       </c>
-      <c r="T14" t="n">
-        <v>0.2266666666666667</v>
-      </c>
-      <c r="U14" t="n">
-        <v>0.2133333333333333</v>
+      <c r="W14" t="n">
+        <v>0.22</v>
       </c>
     </row>
     <row r="15">
@@ -1469,55 +1557,61 @@
         <v>2012</v>
       </c>
       <c r="E15" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.8666593567251463</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.1794529113741501</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.3692332047685616</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.5741766117669469</v>
+      </c>
+      <c r="K15" t="n">
+        <v>9</v>
+      </c>
+      <c r="L15" t="n">
+        <v>9</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="n">
+        <v>6</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="P15" t="n">
         <v>0.9</v>
       </c>
-      <c r="F15" t="n">
-        <v>0.9126315789473685</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.1729535948149485</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.6117757361783286</v>
-      </c>
-      <c r="I15" t="n">
-        <v>8</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>2</v>
-      </c>
-      <c r="L15" t="n">
-        <v>15</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O15" t="n">
-        <v>1</v>
-      </c>
-      <c r="P15" t="n">
+      <c r="Q15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="V15" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="S15" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="T15" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U15" t="n">
-        <v>0.18</v>
+      <c r="W15" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="16">
@@ -1540,55 +1634,61 @@
         <v>2012</v>
       </c>
       <c r="E16" t="n">
-        <v>0.8733333333333334</v>
+        <v>0.8133333333333334</v>
       </c>
       <c r="F16" t="n">
-        <v>0.8826388888888889</v>
+        <v>0.8189572927072927</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1501580774784088</v>
+        <v>0.1780214309692383</v>
       </c>
       <c r="H16" t="n">
-        <v>0.671759307384491</v>
+        <v>0.0711463987827301</v>
       </c>
       <c r="I16" t="n">
-        <v>8</v>
+        <v>2011</v>
       </c>
       <c r="J16" t="n">
+        <v>0.7178729176521301</v>
+      </c>
+      <c r="K16" t="n">
+        <v>10</v>
+      </c>
+      <c r="L16" t="n">
+        <v>12</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>3</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="P16" t="n">
         <v>1</v>
       </c>
-      <c r="K16" t="n">
-        <v>2</v>
-      </c>
-      <c r="L16" t="n">
-        <v>14</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0.8421052631578947</v>
-      </c>
-      <c r="N16" t="n">
+      <c r="Q16" t="n">
+        <v>0.4545454545454545</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
         <v>0.8</v>
       </c>
-      <c r="O16" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0.06666666666666667</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="S16" t="n">
+      <c r="T16" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="V16" t="n">
         <v>0.16</v>
       </c>
-      <c r="T16" t="n">
-        <v>0.1733333333333334</v>
-      </c>
-      <c r="U16" t="n">
-        <v>0.1866666666666667</v>
+      <c r="W16" t="n">
+        <v>0.08000000000000002</v>
       </c>
     </row>
     <row r="17">
@@ -1611,55 +1711,61 @@
         <v>2012</v>
       </c>
       <c r="E17" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="F17" t="n">
-        <v>0.7488677988677989</v>
+        <v>0.6498747984042101</v>
       </c>
       <c r="G17" t="n">
-        <v>0.217466614056738</v>
+        <v>0.2200209291711988</v>
       </c>
       <c r="H17" t="n">
-        <v>0.4996605725769222</v>
+        <v>0.5022939176665918</v>
       </c>
       <c r="I17" t="n">
-        <v>9</v>
+        <v>2011</v>
       </c>
       <c r="J17" t="n">
+        <v>0.4291099085012656</v>
+      </c>
+      <c r="K17" t="n">
+        <v>4</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2</v>
+      </c>
+      <c r="M17" t="n">
         <v>6</v>
       </c>
-      <c r="K17" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" t="n">
-        <v>9</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0.72</v>
-      </c>
       <c r="N17" t="n">
-        <v>0.9</v>
+        <v>13</v>
       </c>
       <c r="O17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="R17" t="n">
         <v>0.6</v>
       </c>
-      <c r="P17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="R17" t="n">
-        <v>0.72</v>
-      </c>
       <c r="S17" t="n">
-        <v>0.19</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="T17" t="n">
-        <v>0.16</v>
+        <v>0.68</v>
       </c>
       <c r="U17" t="n">
-        <v>0.13</v>
+        <v>0.46</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0.5066666666666666</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0.5533333333333333</v>
       </c>
     </row>
     <row r="18">
@@ -1682,55 +1788,61 @@
         <v>2012</v>
       </c>
       <c r="E18" t="n">
-        <v>0.8233333333333334</v>
+        <v>0.7833333333333334</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7257575757575758</v>
+        <v>0.6547619047619048</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1841320532431732</v>
+        <v>0.1973727974555926</v>
       </c>
       <c r="H18" t="n">
-        <v>0.7374566109182709</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>8</v>
+        <v>2011</v>
       </c>
       <c r="J18" t="n">
-        <v>3</v>
+        <v>0.5583540781959282</v>
       </c>
       <c r="K18" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L18" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M18" t="n">
-        <v>0.7619047619047619</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="P18" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V18" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q18" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="R18" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="S18" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="T18" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="U18" t="n">
-        <v>0.2</v>
+      <c r="W18" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="19">
@@ -1753,55 +1865,61 @@
         <v>2012</v>
       </c>
       <c r="E19" t="n">
-        <v>0.9</v>
+        <v>0.8933333333333333</v>
       </c>
       <c r="F19" t="n">
-        <v>0.9003588516746411</v>
+        <v>0.8730680868838764</v>
       </c>
       <c r="G19" t="n">
-        <v>0.1384474904804223</v>
+        <v>0.127770858636771</v>
       </c>
       <c r="H19" t="n">
-        <v>0.7285815117256835</v>
+        <v>0.1237974127607304</v>
       </c>
       <c r="I19" t="n">
-        <v>7</v>
+        <v>2011</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>0.6671975414795391</v>
       </c>
       <c r="K19" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L19" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="M19" t="n">
-        <v>0.8235294117647058</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>0.7</v>
+        <v>6</v>
       </c>
       <c r="O19" t="n">
+        <v>0.6896551724137931</v>
+      </c>
+      <c r="P19" t="n">
         <v>1</v>
       </c>
-      <c r="P19" t="n">
-        <v>0.3</v>
-      </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="R19" t="n">
-        <v>0.88</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>0.21</v>
+        <v>0.6</v>
       </c>
       <c r="T19" t="n">
-        <v>0.24</v>
+        <v>0.64</v>
       </c>
       <c r="U19" t="n">
-        <v>0.27</v>
+        <v>0.18</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="20">
@@ -1832,48 +1950,24 @@
       <c r="G20" t="n">
         <v>0.2155429920581876</v>
       </c>
-      <c r="H20" t="n">
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="n">
         <v>0.214396107376168</v>
       </c>
-      <c r="I20" t="n">
-        <v>8</v>
-      </c>
-      <c r="J20" t="n">
-        <v>6</v>
-      </c>
-      <c r="K20" t="n">
-        <v>2</v>
-      </c>
-      <c r="L20" t="n">
-        <v>9</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="S20" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="T20" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="U20" t="n">
-        <v>0.22</v>
-      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1895,56 +1989,32 @@
         <v>2011</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6733333333333333</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="F21" t="n">
-        <v>0.6533760683760683</v>
+        <v>0.6704761904761904</v>
       </c>
       <c r="G21" t="n">
-        <v>0.3209719999999999</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="I21" t="n">
-        <v>8</v>
-      </c>
+        <v>0.316336</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="n">
-        <v>8</v>
-      </c>
-      <c r="K21" t="n">
-        <v>2</v>
-      </c>
-      <c r="L21" t="n">
-        <v>7</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.6153846153846154</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0.5333333333333333</v>
-      </c>
-      <c r="R21" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="S21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T21" t="n">
-        <v>0.2666666666666667</v>
-      </c>
-      <c r="U21" t="n">
-        <v>0.2333333333333334</v>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1974,48 +2044,24 @@
       <c r="G22" t="n">
         <v>0.312720388174057</v>
       </c>
-      <c r="H22" t="n">
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="n">
         <v>0.004134990740567446</v>
       </c>
-      <c r="I22" t="n">
-        <v>9</v>
-      </c>
-      <c r="J22" t="n">
-        <v>8</v>
-      </c>
-      <c r="K22" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" t="n">
-        <v>7</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0.5294117647058824</v>
-      </c>
-      <c r="P22" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>0.5333333333333333</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="S22" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="T22" t="n">
-        <v>0.1866666666666667</v>
-      </c>
-      <c r="U22" t="n">
-        <v>0.1433333333333333</v>
-      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2040,53 +2086,29 @@
         <v>0.8133333333333334</v>
       </c>
       <c r="F23" t="n">
-        <v>0.798799762329174</v>
+        <v>0.7687098930481283</v>
       </c>
       <c r="G23" t="n">
-        <v>0.1911382389981019</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.1807592812230448</v>
-      </c>
-      <c r="I23" t="n">
-        <v>8</v>
-      </c>
+        <v>0.1949267004583711</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="n">
-        <v>4</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>11</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0.7272727272727273</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="P23" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>0.2666666666666667</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="S23" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="T23" t="n">
-        <v>0.2133333333333334</v>
-      </c>
-      <c r="U23" t="n">
-        <v>0.2066666666666667</v>
-      </c>
+        <v>0.1182109646038034</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2108,56 +2130,32 @@
         <v>2011</v>
       </c>
       <c r="E24" t="n">
-        <v>0.5733333333333333</v>
+        <v>0.5466666666666666</v>
       </c>
       <c r="F24" t="n">
         <v>0.52</v>
       </c>
       <c r="G24" t="n">
-        <v>0.3427203439871637</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>10</v>
-      </c>
+        <v>0.3640205631252207</v>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="n">
-        <v>15</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="N24" t="n">
-        <v>1</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1</v>
-      </c>
-      <c r="R24" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S24" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T24" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="U24" t="n">
-        <v>0.1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2187,48 +2185,24 @@
       <c r="G25" t="n">
         <v>0.2764459795613017</v>
       </c>
-      <c r="H25" t="n">
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="n">
         <v>0.003988136469010892</v>
       </c>
-      <c r="I25" t="n">
-        <v>8</v>
-      </c>
-      <c r="J25" t="n">
-        <v>1</v>
-      </c>
-      <c r="K25" t="n">
-        <v>2</v>
-      </c>
-      <c r="L25" t="n">
-        <v>14</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0.8421052631578947</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="P25" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>0.06666666666666667</v>
-      </c>
-      <c r="R25" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="S25" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="T25" t="n">
-        <v>0.1733333333333334</v>
-      </c>
-      <c r="U25" t="n">
-        <v>0.1866666666666667</v>
-      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2259,46 +2233,52 @@
         <v>0.1831261321893823</v>
       </c>
       <c r="H26" t="n">
+        <v>0.214396107376168</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J26" t="n">
         <v>0.1466912697483659</v>
       </c>
-      <c r="I26" t="n">
-        <v>10</v>
-      </c>
-      <c r="J26" t="n">
-        <v>7</v>
-      </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L26" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M26" t="n">
-        <v>0.7407407407407407</v>
+        <v>4</v>
       </c>
       <c r="N26" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="O26" t="n">
-        <v>0.5882352941176471</v>
+        <v>0.6</v>
       </c>
       <c r="P26" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.4666666666666667</v>
+        <v>0.6</v>
       </c>
       <c r="R26" t="n">
-        <v>0.72</v>
+        <v>0.4</v>
       </c>
       <c r="S26" t="n">
-        <v>0.14</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="T26" t="n">
-        <v>0.09333333333333334</v>
+        <v>0.68</v>
       </c>
       <c r="U26" t="n">
-        <v>0.04666666666666667</v>
+        <v>0.36</v>
+      </c>
+      <c r="V26" t="n">
+        <v>0.3733333333333334</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.3866666666666667</v>
       </c>
     </row>
     <row r="27">
@@ -2321,55 +2301,61 @@
         <v>2012</v>
       </c>
       <c r="E27" t="n">
-        <v>0.8866666666666666</v>
+        <v>0.8400000000000001</v>
       </c>
       <c r="F27" t="n">
-        <v>0.8323841354723708</v>
+        <v>0.8123364859777903</v>
       </c>
       <c r="G27" t="n">
-        <v>0.216776</v>
+        <v>0.231272</v>
       </c>
       <c r="H27" t="n">
-        <v>0.25</v>
+        <v>0.01</v>
       </c>
       <c r="I27" t="n">
-        <v>7</v>
+        <v>2011</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0.23</v>
       </c>
       <c r="K27" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L27" t="n">
         <v>14</v>
       </c>
       <c r="M27" t="n">
-        <v>0.7777777777777778</v>
+        <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="O27" t="n">
-        <v>0.875</v>
+        <v>0.5882352941176471</v>
       </c>
       <c r="P27" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="R27" t="n">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>0.23</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="T27" t="n">
-        <v>0.2533333333333333</v>
+        <v>0.44</v>
       </c>
       <c r="U27" t="n">
-        <v>0.2766666666666667</v>
+        <v>0.28</v>
+      </c>
+      <c r="V27" t="n">
+        <v>0.1866666666666667</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.09333333333333334</v>
       </c>
     </row>
     <row r="28">
@@ -2401,46 +2387,52 @@
         <v>0.2171606421470642</v>
       </c>
       <c r="H28" t="n">
+        <v>0.004134990740567446</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J28" t="n">
         <v>0.03543443605303764</v>
       </c>
-      <c r="I28" t="n">
-        <v>8</v>
-      </c>
-      <c r="J28" t="n">
-        <v>3</v>
-      </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L28" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M28" t="n">
-        <v>0.7619047619047619</v>
+        <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>0.8</v>
+        <v>5</v>
       </c>
       <c r="O28" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.6206896551724138</v>
       </c>
       <c r="P28" t="n">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.2</v>
+        <v>0.4736842105263158</v>
       </c>
       <c r="R28" t="n">
-        <v>0.8</v>
+        <v>0.1</v>
       </c>
       <c r="S28" t="n">
-        <v>0.2</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="T28" t="n">
-        <v>0.2</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="U28" t="n">
-        <v>0.2</v>
+        <v>0.27</v>
+      </c>
+      <c r="V28" t="n">
+        <v>0.2133333333333333</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.1566666666666667</v>
       </c>
     </row>
     <row r="29">
@@ -2463,54 +2455,60 @@
         <v>2012</v>
       </c>
       <c r="E29" t="n">
-        <v>0.8266666666666667</v>
+        <v>0.8200000000000001</v>
       </c>
       <c r="F29" t="n">
-        <v>0.8286247086247086</v>
+        <v>0.8166117216117216</v>
       </c>
       <c r="G29" t="n">
-        <v>0.1741227916710872</v>
+        <v>0.1722255190839223</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1691485916788619</v>
+        <v>0.1182109646038034</v>
       </c>
       <c r="I29" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.1630865851576783</v>
+      </c>
+      <c r="K29" t="n">
         <v>9</v>
       </c>
-      <c r="J29" t="n">
+      <c r="L29" t="n">
         <v>4</v>
       </c>
-      <c r="K29" t="n">
+      <c r="M29" t="n">
         <v>1</v>
       </c>
-      <c r="L29" t="n">
+      <c r="N29" t="n">
         <v>11</v>
       </c>
-      <c r="M29" t="n">
+      <c r="O29" t="n">
         <v>0.7826086956521739</v>
       </c>
-      <c r="N29" t="n">
+      <c r="P29" t="n">
         <v>0.9</v>
       </c>
-      <c r="O29" t="n">
+      <c r="Q29" t="n">
         <v>0.6923076923076923</v>
       </c>
-      <c r="P29" t="n">
+      <c r="R29" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q29" t="n">
+      <c r="S29" t="n">
         <v>0.2666666666666667</v>
       </c>
-      <c r="R29" t="n">
+      <c r="T29" t="n">
         <v>0.8</v>
       </c>
-      <c r="S29" t="n">
+      <c r="U29" t="n">
         <v>0.15</v>
       </c>
-      <c r="T29" t="n">
+      <c r="V29" t="n">
         <v>0.1333333333333334</v>
       </c>
-      <c r="U29" t="n">
+      <c r="W29" t="n">
         <v>0.1166666666666667</v>
       </c>
     </row>
@@ -2546,42 +2544,48 @@
         <v>0</v>
       </c>
       <c r="I30" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
         <v>10</v>
       </c>
-      <c r="J30" t="n">
+      <c r="L30" t="n">
         <v>15</v>
       </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
       <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
         <v>0.5714285714285714</v>
       </c>
-      <c r="N30" t="n">
+      <c r="P30" t="n">
         <v>1</v>
       </c>
-      <c r="O30" t="n">
+      <c r="Q30" t="n">
         <v>0.4</v>
       </c>
-      <c r="P30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" t="n">
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="n">
         <v>1</v>
       </c>
-      <c r="R30" t="n">
+      <c r="T30" t="n">
         <v>0.4</v>
       </c>
-      <c r="S30" t="n">
+      <c r="U30" t="n">
         <v>0.3</v>
       </c>
-      <c r="T30" t="n">
+      <c r="V30" t="n">
         <v>0.2</v>
       </c>
-      <c r="U30" t="n">
+      <c r="W30" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -2614,46 +2618,52 @@
         <v>0.2019680095014026</v>
       </c>
       <c r="H31" t="n">
+        <v>0.003988136469010892</v>
+      </c>
+      <c r="I31" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J31" t="n">
         <v>0.02090703665427157</v>
       </c>
-      <c r="I31" t="n">
+      <c r="K31" t="n">
         <v>9</v>
       </c>
-      <c r="J31" t="n">
-        <v>2</v>
-      </c>
-      <c r="K31" t="n">
+      <c r="L31" t="n">
+        <v>7</v>
+      </c>
+      <c r="M31" t="n">
         <v>1</v>
       </c>
-      <c r="L31" t="n">
-        <v>13</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0.8571428571428571</v>
-      </c>
       <c r="N31" t="n">
+        <v>8</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0.6923076923076923</v>
+      </c>
+      <c r="P31" t="n">
         <v>0.9</v>
       </c>
-      <c r="O31" t="n">
-        <v>0.8181818181818182</v>
-      </c>
-      <c r="P31" t="n">
+      <c r="Q31" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="R31" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q31" t="n">
-        <v>0.1333333333333333</v>
-      </c>
-      <c r="R31" t="n">
-        <v>0.88</v>
-      </c>
       <c r="S31" t="n">
-        <v>0.11</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="T31" t="n">
-        <v>0.1066666666666667</v>
+        <v>0.68</v>
       </c>
       <c r="U31" t="n">
-        <v>0.1033333333333333</v>
+        <v>0.21</v>
+      </c>
+      <c r="V31" t="n">
+        <v>0.1733333333333333</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0.1366666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -2689,7 +2699,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.603</v>
+        <v>0.576</v>
       </c>
     </row>
     <row r="3">
@@ -2699,7 +2709,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.782</v>
+        <v>0.753</v>
       </c>
     </row>
     <row r="4">
@@ -2709,7 +2719,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.638</v>
+        <v>0.636</v>
       </c>
     </row>
     <row r="5">
@@ -2719,7 +2729,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.627</v>
+        <v>0.658</v>
       </c>
     </row>
     <row r="6">
@@ -2729,7 +2739,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.646</v>
       </c>
     </row>
     <row r="7">
@@ -2739,7 +2749,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.711</v>
+        <v>0.716</v>
       </c>
     </row>
   </sheetData>
@@ -2815,25 +2825,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.603</v>
+        <v>0.576</v>
       </c>
       <c r="D2" t="n">
-        <v>0.658</v>
+        <v>0.499</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.767</v>
       </c>
       <c r="F2" t="n">
-        <v>0.533</v>
+        <v>0.41</v>
       </c>
       <c r="G2" t="n">
-        <v>0.067</v>
+        <v>0.233</v>
       </c>
       <c r="H2" t="n">
-        <v>0.644</v>
+        <v>0.756</v>
       </c>
       <c r="I2" t="n">
-        <v>0.182</v>
+        <v>0.338</v>
       </c>
     </row>
     <row r="3">
@@ -2848,25 +2858,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.782</v>
+        <v>0.753</v>
       </c>
       <c r="D3" t="n">
-        <v>0.756</v>
+        <v>0.705</v>
       </c>
       <c r="E3" t="n">
-        <v>0.867</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.735</v>
+        <v>0.549</v>
       </c>
       <c r="G3" t="n">
-        <v>0.133</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0.333</v>
+        <v>0.578</v>
       </c>
       <c r="I3" t="n">
-        <v>0.173</v>
+        <v>0.116</v>
       </c>
     </row>
     <row r="4">
@@ -2881,25 +2891,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.638</v>
+        <v>0.636</v>
       </c>
       <c r="D4" t="n">
-        <v>0.637</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="F4" t="n">
-        <v>0.505</v>
+        <v>0.449</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H4" t="n">
-        <v>0.644</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>0.209</v>
+        <v>0.298</v>
       </c>
     </row>
     <row r="5">
@@ -2914,25 +2924,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.627</v>
+        <v>0.658</v>
       </c>
       <c r="D5" t="n">
-        <v>0.648</v>
+        <v>0.531</v>
       </c>
       <c r="E5" t="n">
-        <v>0.867</v>
+        <v>0.667</v>
       </c>
       <c r="F5" t="n">
+        <v>0.509</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="H5" t="n">
         <v>0.533</v>
       </c>
-      <c r="G5" t="n">
-        <v>0.133</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.556</v>
-      </c>
       <c r="I5" t="n">
-        <v>0.218</v>
+        <v>0.373</v>
       </c>
     </row>
     <row r="6">
@@ -2947,25 +2957,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.646</v>
       </c>
       <c r="D6" t="n">
-        <v>0.721</v>
+        <v>0.607</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.967</v>
       </c>
       <c r="F6" t="n">
-        <v>0.645</v>
+        <v>0.445</v>
       </c>
       <c r="G6" t="n">
-        <v>0.067</v>
+        <v>0.033</v>
       </c>
       <c r="H6" t="n">
-        <v>0.511</v>
+        <v>0.822</v>
       </c>
       <c r="I6" t="n">
-        <v>0.156</v>
+        <v>0.191</v>
       </c>
     </row>
     <row r="7">
@@ -2980,25 +2990,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.711</v>
+        <v>0.716</v>
       </c>
       <c r="D7" t="n">
-        <v>0.731</v>
+        <v>0.595</v>
       </c>
       <c r="E7" t="n">
-        <v>0.867</v>
+        <v>0.833</v>
       </c>
       <c r="F7" t="n">
-        <v>0.67</v>
+        <v>0.523</v>
       </c>
       <c r="G7" t="n">
-        <v>0.133</v>
+        <v>0.167</v>
       </c>
       <c r="H7" t="n">
-        <v>0.378</v>
+        <v>0.644</v>
       </c>
       <c r="I7" t="n">
-        <v>0.182</v>
+        <v>0.262</v>
       </c>
     </row>
   </sheetData>
@@ -3044,7 +3054,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.603</v>
+        <v>0.576</v>
       </c>
     </row>
     <row r="3">
@@ -3054,7 +3064,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.782</v>
+        <v>0.753</v>
       </c>
     </row>
     <row r="4">
@@ -3064,7 +3074,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.638</v>
+        <v>0.636</v>
       </c>
     </row>
     <row r="5">
@@ -3074,7 +3084,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.627</v>
+        <v>0.658</v>
       </c>
     </row>
     <row r="6">
@@ -3084,7 +3094,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.646</v>
       </c>
     </row>
     <row r="7">
@@ -3094,7 +3104,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.711</v>
+        <v>0.716</v>
       </c>
     </row>
     <row r="8">
@@ -3109,7 +3119,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.57</v>
+        <v>0.5570000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -3139,7 +3149,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.82</v>
+        <v>0.8169999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -3149,7 +3159,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.78</v>
+        <v>0.787</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Rerun the pre-crisis check on the corrected data (seed 27)
Same fixes as the seed 42 worktree: credit_gap_missing dropped at load in rt2b,
nfa_g replaced by nfa_gdp, 'crisis' excluded from micro_cols, threshold metrics
left empty (one test year has no evaluated predecessor), and the A46
falsification baseline added. rt2a/rt2b returned to tools/run_pipeline.py.

The falsification rule scores AUROC 1.000 here too.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/results/12a_gran/results_12a_isolate_gran_final.xlsx
+++ b/outputs/results/12a_gran/results_12a_isolate_gran_final.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:W31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,65 +462,75 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>threshold_from_year</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>test_optimal_threshold</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>tp</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>fp</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>fn</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>tn</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>f1</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>precision</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>miss_rate</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>false_alarm_rate</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>accuracy</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>loss_07</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>loss_08</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>loss_09</t>
         </is>
@@ -555,46 +565,52 @@
         <v>0.3302682062847694</v>
       </c>
       <c r="H2" t="n">
+        <v>0.4134512387890711</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J2" t="n">
         <v>0.01663706238879454</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L2" t="n">
         <v>10</v>
       </c>
-      <c r="J2" t="n">
-        <v>15</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
       <c r="M2" t="n">
-        <v>0.5714285714285714</v>
+        <v>4</v>
       </c>
       <c r="N2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O2" t="n">
-        <v>0.4</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>0.375</v>
       </c>
       <c r="R2" t="n">
         <v>0.4</v>
       </c>
       <c r="S2" t="n">
-        <v>0.3</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="T2" t="n">
-        <v>0.2</v>
+        <v>0.44</v>
       </c>
       <c r="U2" t="n">
-        <v>0.1</v>
+        <v>0.48</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.4533333333333334</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.4266666666666667</v>
       </c>
     </row>
     <row r="3">
@@ -617,55 +633,61 @@
         <v>2010</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5166666666666667</v>
+        <v>0.4266666666666666</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4386503256468932</v>
+        <v>0.3718049599702581</v>
       </c>
       <c r="G3" t="n">
-        <v>0.247256</v>
+        <v>0.268484</v>
       </c>
       <c r="H3" t="n">
-        <v>0.32</v>
+        <v>0.08</v>
       </c>
       <c r="I3" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="K3" t="n">
         <v>10</v>
       </c>
-      <c r="J3" t="n">
-        <v>13</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
       <c r="L3" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6060606060606061</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" t="n">
-        <v>0.4347826086956522</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
       <c r="Q3" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.4</v>
       </c>
       <c r="R3" t="n">
-        <v>0.48</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0.26</v>
+        <v>1</v>
       </c>
       <c r="T3" t="n">
-        <v>0.1733333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="U3" t="n">
-        <v>0.08666666666666667</v>
+        <v>0.3</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="4">
@@ -697,46 +719,52 @@
         <v>0.3515652120113373</v>
       </c>
       <c r="H4" t="n">
+        <v>0.01242134533822536</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J4" t="n">
         <v>0.3752442896366119</v>
       </c>
-      <c r="I4" t="n">
+      <c r="K4" t="n">
         <v>10</v>
       </c>
-      <c r="J4" t="n">
-        <v>12</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
       <c r="L4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="M4" t="n">
-        <v>0.625</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="n">
-        <v>0.4545454545454545</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
       <c r="Q4" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="R4" t="n">
-        <v>0.52</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>0.24</v>
+        <v>1</v>
       </c>
       <c r="T4" t="n">
-        <v>0.16</v>
+        <v>0.4</v>
       </c>
       <c r="U4" t="n">
-        <v>0.08000000000000002</v>
+        <v>0.3</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="5">
@@ -759,55 +787,61 @@
         <v>2010</v>
       </c>
       <c r="E5" t="n">
-        <v>0.44</v>
+        <v>0.4066666666666667</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3808868908868909</v>
+        <v>0.358526601481407</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4000947300528722</v>
+        <v>0.4141745764180273</v>
       </c>
       <c r="H5" t="n">
-        <v>0.03566289372715235</v>
+        <v>0.3151653653242443</v>
       </c>
       <c r="I5" t="n">
-        <v>10</v>
+        <v>2009</v>
       </c>
       <c r="J5" t="n">
-        <v>14</v>
+        <v>0.05811293921009648</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5882352941176471</v>
+        <v>4</v>
       </c>
       <c r="N5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O5" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.48</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="R5" t="n">
-        <v>0.44</v>
+        <v>0.4</v>
       </c>
       <c r="S5" t="n">
-        <v>0.28</v>
+        <v>0.6</v>
       </c>
       <c r="T5" t="n">
-        <v>0.1866666666666667</v>
+        <v>0.48</v>
       </c>
       <c r="U5" t="n">
-        <v>0.09333333333333334</v>
+        <v>0.46</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.4400000000000001</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.42</v>
       </c>
     </row>
     <row r="6">
@@ -830,55 +864,61 @@
         <v>2010</v>
       </c>
       <c r="E6" t="n">
-        <v>0.45</v>
+        <v>0.43</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3988636363636364</v>
+        <v>0.3757575757575758</v>
       </c>
       <c r="G6" t="n">
-        <v>0.379083972587156</v>
+        <v>0.3813672950534979</v>
       </c>
       <c r="H6" t="n">
-        <v>0.420814479638009</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.4208144796380091</v>
+      </c>
+      <c r="K6" t="n">
         <v>10</v>
       </c>
-      <c r="J6" t="n">
-        <v>14</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
       <c r="L6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P6" t="n">
         <v>1</v>
       </c>
-      <c r="M6" t="n">
-        <v>0.5882352941176471</v>
-      </c>
-      <c r="N6" t="n">
+      <c r="Q6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
         <v>1</v>
       </c>
-      <c r="O6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.9333333333333333</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.28</v>
-      </c>
       <c r="T6" t="n">
-        <v>0.1866666666666667</v>
+        <v>0.4</v>
       </c>
       <c r="U6" t="n">
-        <v>0.09333333333333334</v>
+        <v>0.3</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="7">
@@ -910,45 +950,51 @@
         <v>0.3083624220446608</v>
       </c>
       <c r="H7" t="n">
+        <v>0.04470937183400933</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J7" t="n">
         <v>0.1188634608818508</v>
       </c>
-      <c r="I7" t="n">
+      <c r="K7" t="n">
         <v>10</v>
       </c>
-      <c r="J7" t="n">
+      <c r="L7" t="n">
         <v>12</v>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
         <v>3</v>
       </c>
-      <c r="M7" t="n">
+      <c r="O7" t="n">
         <v>0.625</v>
       </c>
-      <c r="N7" t="n">
+      <c r="P7" t="n">
         <v>1</v>
       </c>
-      <c r="O7" t="n">
+      <c r="Q7" t="n">
         <v>0.4545454545454545</v>
       </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
         <v>0.8</v>
       </c>
-      <c r="R7" t="n">
+      <c r="T7" t="n">
         <v>0.52</v>
       </c>
-      <c r="S7" t="n">
+      <c r="U7" t="n">
         <v>0.24</v>
       </c>
-      <c r="T7" t="n">
+      <c r="V7" t="n">
         <v>0.16</v>
       </c>
-      <c r="U7" t="n">
+      <c r="W7" t="n">
         <v>0.08000000000000002</v>
       </c>
     </row>
@@ -972,55 +1018,61 @@
         <v>2011</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.66</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6510926399545325</v>
+        <v>0.6472464861083786</v>
       </c>
       <c r="G8" t="n">
-        <v>0.24142315899945</v>
+        <v>0.2423127877206176</v>
       </c>
       <c r="H8" t="n">
-        <v>0.479564160817484</v>
+        <v>0.01663706238879454</v>
       </c>
       <c r="I8" t="n">
-        <v>9</v>
+        <v>2010</v>
       </c>
       <c r="J8" t="n">
-        <v>9</v>
+        <v>0.4819643744241356</v>
       </c>
       <c r="K8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" t="n">
+        <v>15</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P8" t="n">
         <v>1</v>
       </c>
-      <c r="L8" t="n">
-        <v>6</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.6428571428571429</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W8" t="n">
         <v>0.1</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="U8" t="n">
-        <v>0.15</v>
       </c>
     </row>
     <row r="9">
@@ -1043,55 +1095,61 @@
         <v>2011</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6533333333333333</v>
+        <v>0.6733333333333333</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5856434793276898</v>
+        <v>0.5829411764705882</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2230026896503645</v>
+        <v>0.216325776017708</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3845475210954841</v>
+        <v>0.34</v>
       </c>
       <c r="I9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.4164346471106978</v>
+      </c>
+      <c r="K9" t="n">
         <v>10</v>
       </c>
-      <c r="J9" t="n">
-        <v>10</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
       <c r="L9" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="M9" t="n">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
+        <v>4</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.6451612903225806</v>
+      </c>
+      <c r="P9" t="n">
         <v>1</v>
       </c>
-      <c r="O9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
       <c r="Q9" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="R9" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0.2</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="T9" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="U9" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.22</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.1466666666666667</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.07333333333333333</v>
       </c>
     </row>
     <row r="10">
@@ -1114,55 +1172,61 @@
         <v>2011</v>
       </c>
       <c r="E10" t="n">
-        <v>0.7533333333333334</v>
+        <v>0.8200000000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6665909090909091</v>
+        <v>0.7082815713698066</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2561646401882172</v>
+        <v>0.2257847040891647</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1051026284694672</v>
+        <v>0.3752442896366119</v>
       </c>
       <c r="I10" t="n">
-        <v>8</v>
+        <v>2010</v>
       </c>
       <c r="J10" t="n">
+        <v>0.1286037415266037</v>
+      </c>
+      <c r="K10" t="n">
         <v>4</v>
       </c>
-      <c r="K10" t="n">
-        <v>2</v>
-      </c>
       <c r="L10" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
-        <v>0.7272727272727273</v>
+        <v>6</v>
       </c>
       <c r="N10" t="n">
-        <v>0.8</v>
+        <v>12</v>
       </c>
       <c r="O10" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4705882352941176</v>
       </c>
       <c r="P10" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="S10" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q10" t="n">
-        <v>0.2666666666666667</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0.22</v>
-      </c>
       <c r="T10" t="n">
-        <v>0.2133333333333334</v>
+        <v>0.64</v>
       </c>
       <c r="U10" t="n">
-        <v>0.2066666666666667</v>
+        <v>0.48</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -1185,55 +1249,61 @@
         <v>2011</v>
       </c>
       <c r="E11" t="n">
-        <v>0.7</v>
+        <v>0.5466666666666666</v>
       </c>
       <c r="F11" t="n">
-        <v>0.6983467023172906</v>
+        <v>0.5763372893016856</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2332489029133263</v>
+        <v>0.2485602109792572</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4910117331747179</v>
+        <v>0.05811293921009648</v>
       </c>
       <c r="I11" t="n">
-        <v>7</v>
+        <v>2010</v>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>0.1611375775235966</v>
       </c>
       <c r="K11" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="M11" t="n">
-        <v>0.6363636363636364</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="P11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U11" t="n">
         <v>0.3</v>
       </c>
-      <c r="Q11" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="T11" t="n">
-        <v>0.3066666666666666</v>
-      </c>
-      <c r="U11" t="n">
-        <v>0.3033333333333333</v>
+      <c r="V11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="12">
@@ -1262,49 +1332,55 @@
         <v>0.4340909090909091</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2656166240652603</v>
+        <v>0.2555023364787536</v>
       </c>
       <c r="H12" t="n">
-        <v>0.3287671232876714</v>
+        <v>0.4208144796380091</v>
       </c>
       <c r="I12" t="n">
-        <v>10</v>
+        <v>2010</v>
       </c>
       <c r="J12" t="n">
-        <v>12</v>
+        <v>0.3287671232876713</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L12" t="n">
         <v>3</v>
       </c>
       <c r="M12" t="n">
-        <v>0.625</v>
+        <v>9</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="O12" t="n">
-        <v>0.4545454545454545</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.8</v>
+        <v>0.25</v>
       </c>
       <c r="R12" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="T12" t="n">
         <v>0.52</v>
       </c>
-      <c r="S12" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="T12" t="n">
-        <v>0.16</v>
-      </c>
       <c r="U12" t="n">
-        <v>0.08000000000000002</v>
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.7600000000000001</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.8300000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -1327,55 +1403,61 @@
         <v>2011</v>
       </c>
       <c r="E13" t="n">
-        <v>0.88</v>
+        <v>0.8200000000000001</v>
       </c>
       <c r="F13" t="n">
-        <v>0.8263383838383839</v>
+        <v>0.7076839826839826</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2879982548758644</v>
+        <v>0.2131499327466811</v>
       </c>
       <c r="H13" t="n">
-        <v>0.005595969106936115</v>
+        <v>0.1188634608818508</v>
       </c>
       <c r="I13" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.1006472771555486</v>
+      </c>
+      <c r="K13" t="n">
         <v>9</v>
       </c>
-      <c r="J13" t="n">
-        <v>3</v>
-      </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
+        <v>5</v>
+      </c>
+      <c r="M13" t="n">
         <v>1</v>
       </c>
-      <c r="L13" t="n">
-        <v>12</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.8181818181818182</v>
-      </c>
       <c r="N13" t="n">
-        <v>0.9</v>
+        <v>10</v>
       </c>
       <c r="O13" t="n">
         <v>0.75</v>
       </c>
       <c r="P13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="R13" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0.84</v>
-      </c>
       <c r="S13" t="n">
-        <v>0.13</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="T13" t="n">
-        <v>0.12</v>
+        <v>0.76</v>
       </c>
       <c r="U13" t="n">
-        <v>0.11</v>
+        <v>0.17</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.1466666666666667</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.1233333333333334</v>
       </c>
     </row>
     <row r="14">
@@ -1404,48 +1486,54 @@
         <v>0.7106672494172493</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2015931568180839</v>
+        <v>0.2012769745631847</v>
       </c>
       <c r="H14" t="n">
-        <v>0.4839371869283402</v>
+        <v>0.4819643744241356</v>
       </c>
       <c r="I14" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.4843801213676752</v>
+      </c>
+      <c r="K14" t="n">
         <v>8</v>
       </c>
-      <c r="J14" t="n">
+      <c r="L14" t="n">
         <v>5</v>
       </c>
-      <c r="K14" t="n">
+      <c r="M14" t="n">
         <v>2</v>
       </c>
-      <c r="L14" t="n">
+      <c r="N14" t="n">
         <v>10</v>
       </c>
-      <c r="M14" t="n">
+      <c r="O14" t="n">
         <v>0.6956521739130435</v>
       </c>
-      <c r="N14" t="n">
+      <c r="P14" t="n">
         <v>0.8</v>
       </c>
-      <c r="O14" t="n">
+      <c r="Q14" t="n">
         <v>0.6153846153846154</v>
       </c>
-      <c r="P14" t="n">
+      <c r="R14" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="S14" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="R14" t="n">
+      <c r="T14" t="n">
         <v>0.72</v>
       </c>
-      <c r="S14" t="n">
+      <c r="U14" t="n">
         <v>0.24</v>
       </c>
-      <c r="T14" t="n">
+      <c r="V14" t="n">
         <v>0.2266666666666667</v>
       </c>
-      <c r="U14" t="n">
+      <c r="W14" t="n">
         <v>0.2133333333333333</v>
       </c>
     </row>
@@ -1469,55 +1557,61 @@
         <v>2012</v>
       </c>
       <c r="E15" t="n">
+        <v>0.9066666666666667</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.9192307692307692</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.1500343333125837</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.4164346471106978</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.5556365800040225</v>
+      </c>
+      <c r="K15" t="n">
+        <v>9</v>
+      </c>
+      <c r="L15" t="n">
+        <v>4</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="n">
+        <v>11</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.7826086956521739</v>
+      </c>
+      <c r="P15" t="n">
         <v>0.9</v>
       </c>
-      <c r="F15" t="n">
-        <v>0.9126315789473685</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.1729535948149485</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.6117757361783286</v>
-      </c>
-      <c r="I15" t="n">
-        <v>8</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>2</v>
-      </c>
-      <c r="L15" t="n">
-        <v>15</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="N15" t="n">
+      <c r="Q15" t="n">
+        <v>0.6923076923076923</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="T15" t="n">
         <v>0.8</v>
       </c>
-      <c r="O15" t="n">
-        <v>1</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="S15" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="T15" t="n">
-        <v>0.16</v>
-      </c>
       <c r="U15" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0.1333333333333334</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0.1166666666666667</v>
       </c>
     </row>
     <row r="16">
@@ -1540,55 +1634,61 @@
         <v>2012</v>
       </c>
       <c r="E16" t="n">
-        <v>0.8733333333333334</v>
+        <v>0.8266666666666667</v>
       </c>
       <c r="F16" t="n">
-        <v>0.8826388888888889</v>
+        <v>0.8496212121212121</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1501580774784088</v>
+        <v>0.1742675006389618</v>
       </c>
       <c r="H16" t="n">
-        <v>0.671759307384491</v>
+        <v>0.1286037415266037</v>
       </c>
       <c r="I16" t="n">
-        <v>8</v>
+        <v>2011</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>0.6440360546112061</v>
       </c>
       <c r="K16" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L16" t="n">
         <v>14</v>
       </c>
       <c r="M16" t="n">
-        <v>0.8421052631578947</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="O16" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.5882352941176471</v>
       </c>
       <c r="P16" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="R16" t="n">
-        <v>0.88</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>0.16</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="T16" t="n">
-        <v>0.1733333333333334</v>
+        <v>0.44</v>
       </c>
       <c r="U16" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="V16" t="n">
         <v>0.1866666666666667</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0.09333333333333334</v>
       </c>
     </row>
     <row r="17">
@@ -1611,55 +1711,61 @@
         <v>2012</v>
       </c>
       <c r="E17" t="n">
-        <v>0.74</v>
+        <v>0.7266666666666667</v>
       </c>
       <c r="F17" t="n">
-        <v>0.7488677988677989</v>
+        <v>0.5715060378218273</v>
       </c>
       <c r="G17" t="n">
-        <v>0.217466614056738</v>
+        <v>0.3243709675850251</v>
       </c>
       <c r="H17" t="n">
-        <v>0.4996605725769222</v>
+        <v>0.1611375775235966</v>
       </c>
       <c r="I17" t="n">
-        <v>9</v>
+        <v>2011</v>
       </c>
       <c r="J17" t="n">
-        <v>6</v>
+        <v>0.6624341298176242</v>
       </c>
       <c r="K17" t="n">
+        <v>10</v>
+      </c>
+      <c r="L17" t="n">
+        <v>15</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P17" t="n">
         <v>1</v>
-      </c>
-      <c r="L17" t="n">
-        <v>9</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="N17" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="P17" t="n">
-        <v>0.1</v>
       </c>
       <c r="Q17" t="n">
         <v>0.4</v>
       </c>
       <c r="R17" t="n">
-        <v>0.72</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>0.19</v>
+        <v>1</v>
       </c>
       <c r="T17" t="n">
-        <v>0.16</v>
+        <v>0.4</v>
       </c>
       <c r="U17" t="n">
-        <v>0.13</v>
+        <v>0.3</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="18">
@@ -1682,55 +1788,61 @@
         <v>2012</v>
       </c>
       <c r="E18" t="n">
-        <v>0.8233333333333334</v>
+        <v>0.7833333333333334</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7257575757575758</v>
+        <v>0.6547619047619048</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1841320532431732</v>
+        <v>0.1979003318156931</v>
       </c>
       <c r="H18" t="n">
-        <v>0.7374566109182709</v>
+        <v>0.3287671232876713</v>
       </c>
       <c r="I18" t="n">
-        <v>8</v>
+        <v>2011</v>
       </c>
       <c r="J18" t="n">
-        <v>3</v>
+        <v>0.5537422622397292</v>
       </c>
       <c r="K18" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L18" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M18" t="n">
-        <v>0.7619047619047619</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>0.8</v>
+        <v>4</v>
       </c>
       <c r="O18" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.6451612903225806</v>
       </c>
       <c r="P18" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.2</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="R18" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>0.2</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="T18" t="n">
-        <v>0.2</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="U18" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
+      </c>
+      <c r="V18" t="n">
+        <v>0.1466666666666667</v>
+      </c>
+      <c r="W18" t="n">
+        <v>0.07333333333333333</v>
       </c>
     </row>
     <row r="19">
@@ -1753,55 +1865,61 @@
         <v>2012</v>
       </c>
       <c r="E19" t="n">
-        <v>0.9</v>
+        <v>0.8800000000000001</v>
       </c>
       <c r="F19" t="n">
-        <v>0.9003588516746411</v>
+        <v>0.8852704678362574</v>
       </c>
       <c r="G19" t="n">
-        <v>0.1384474904804223</v>
+        <v>0.1518873133726742</v>
       </c>
       <c r="H19" t="n">
-        <v>0.7285815117256835</v>
+        <v>0.1006472771555486</v>
       </c>
       <c r="I19" t="n">
-        <v>7</v>
+        <v>2011</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>0.6649504080561119</v>
       </c>
       <c r="K19" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L19" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M19" t="n">
-        <v>0.8235294117647058</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>0.7</v>
+        <v>5</v>
       </c>
       <c r="O19" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="P19" t="n">
         <v>1</v>
       </c>
-      <c r="P19" t="n">
-        <v>0.3</v>
-      </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="R19" t="n">
-        <v>0.88</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>0.21</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="T19" t="n">
-        <v>0.24</v>
+        <v>0.6</v>
       </c>
       <c r="U19" t="n">
-        <v>0.27</v>
+        <v>0.2</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="20">
@@ -1832,48 +1950,24 @@
       <c r="G20" t="n">
         <v>0.2155429920581876</v>
       </c>
-      <c r="H20" t="n">
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="n">
         <v>0.214396107376168</v>
       </c>
-      <c r="I20" t="n">
-        <v>8</v>
-      </c>
-      <c r="J20" t="n">
-        <v>6</v>
-      </c>
-      <c r="K20" t="n">
-        <v>2</v>
-      </c>
-      <c r="L20" t="n">
-        <v>9</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="S20" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="T20" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="U20" t="n">
-        <v>0.22</v>
-      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1895,56 +1989,32 @@
         <v>2011</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6733333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F21" t="n">
-        <v>0.6533760683760683</v>
+        <v>0.6133333333333333</v>
       </c>
       <c r="G21" t="n">
-        <v>0.3209719999999999</v>
-      </c>
-      <c r="H21" t="n">
+        <v>0.315916</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="n">
         <v>0.02</v>
       </c>
-      <c r="I21" t="n">
-        <v>8</v>
-      </c>
-      <c r="J21" t="n">
-        <v>8</v>
-      </c>
-      <c r="K21" t="n">
-        <v>2</v>
-      </c>
-      <c r="L21" t="n">
-        <v>7</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.6153846153846154</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0.5333333333333333</v>
-      </c>
-      <c r="R21" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="S21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T21" t="n">
-        <v>0.2666666666666667</v>
-      </c>
-      <c r="U21" t="n">
-        <v>0.2333333333333334</v>
-      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1974,48 +2044,24 @@
       <c r="G22" t="n">
         <v>0.312720388174057</v>
       </c>
-      <c r="H22" t="n">
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="n">
         <v>0.004134990740567446</v>
       </c>
-      <c r="I22" t="n">
-        <v>9</v>
-      </c>
-      <c r="J22" t="n">
-        <v>8</v>
-      </c>
-      <c r="K22" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" t="n">
-        <v>7</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0.5294117647058824</v>
-      </c>
-      <c r="P22" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>0.5333333333333333</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="S22" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="T22" t="n">
-        <v>0.1866666666666667</v>
-      </c>
-      <c r="U22" t="n">
-        <v>0.1433333333333333</v>
-      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2037,56 +2083,32 @@
         <v>2011</v>
       </c>
       <c r="E23" t="n">
-        <v>0.8133333333333334</v>
+        <v>0.8066666666666666</v>
       </c>
       <c r="F23" t="n">
-        <v>0.798799762329174</v>
+        <v>0.7274367299367299</v>
       </c>
       <c r="G23" t="n">
-        <v>0.1911382389981019</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.1807592812230448</v>
-      </c>
-      <c r="I23" t="n">
-        <v>8</v>
-      </c>
+        <v>0.1916400525937622</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="n">
-        <v>4</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>11</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0.7272727272727273</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="P23" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>0.2666666666666667</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="S23" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="T23" t="n">
-        <v>0.2133333333333334</v>
-      </c>
-      <c r="U23" t="n">
-        <v>0.2066666666666667</v>
-      </c>
+        <v>0.1542737257044433</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2116,48 +2138,24 @@
       <c r="G24" t="n">
         <v>0.3427203439871637</v>
       </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>10</v>
-      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="n">
-        <v>15</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="N24" t="n">
-        <v>1</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1</v>
-      </c>
-      <c r="R24" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S24" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T24" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="U24" t="n">
-        <v>0.1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2187,48 +2185,24 @@
       <c r="G25" t="n">
         <v>0.2764459795613017</v>
       </c>
-      <c r="H25" t="n">
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="n">
         <v>0.003988136469010892</v>
       </c>
-      <c r="I25" t="n">
-        <v>8</v>
-      </c>
-      <c r="J25" t="n">
-        <v>1</v>
-      </c>
-      <c r="K25" t="n">
-        <v>2</v>
-      </c>
-      <c r="L25" t="n">
-        <v>14</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0.8421052631578947</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="P25" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>0.06666666666666667</v>
-      </c>
-      <c r="R25" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="S25" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="T25" t="n">
-        <v>0.1733333333333334</v>
-      </c>
-      <c r="U25" t="n">
-        <v>0.1866666666666667</v>
-      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2259,46 +2233,52 @@
         <v>0.1831261321893823</v>
       </c>
       <c r="H26" t="n">
+        <v>0.214396107376168</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J26" t="n">
         <v>0.1466912697483659</v>
       </c>
-      <c r="I26" t="n">
-        <v>10</v>
-      </c>
-      <c r="J26" t="n">
-        <v>7</v>
-      </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L26" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M26" t="n">
-        <v>0.7407407407407407</v>
+        <v>4</v>
       </c>
       <c r="N26" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="O26" t="n">
-        <v>0.5882352941176471</v>
+        <v>0.6</v>
       </c>
       <c r="P26" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.4666666666666667</v>
+        <v>0.6</v>
       </c>
       <c r="R26" t="n">
-        <v>0.72</v>
+        <v>0.4</v>
       </c>
       <c r="S26" t="n">
-        <v>0.14</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="T26" t="n">
-        <v>0.09333333333333334</v>
+        <v>0.68</v>
       </c>
       <c r="U26" t="n">
-        <v>0.04666666666666667</v>
+        <v>0.36</v>
+      </c>
+      <c r="V26" t="n">
+        <v>0.3733333333333334</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.3866666666666667</v>
       </c>
     </row>
     <row r="27">
@@ -2321,55 +2301,61 @@
         <v>2012</v>
       </c>
       <c r="E27" t="n">
-        <v>0.8866666666666666</v>
+        <v>0.8099999999999999</v>
       </c>
       <c r="F27" t="n">
-        <v>0.8323841354723708</v>
+        <v>0.8004670329670329</v>
       </c>
       <c r="G27" t="n">
-        <v>0.216776</v>
+        <v>0.22474</v>
       </c>
       <c r="H27" t="n">
-        <v>0.25</v>
+        <v>0.02</v>
       </c>
       <c r="I27" t="n">
-        <v>7</v>
+        <v>2011</v>
       </c>
       <c r="J27" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="K27" t="n">
+        <v>9</v>
+      </c>
+      <c r="L27" t="n">
+        <v>12</v>
+      </c>
+      <c r="M27" t="n">
         <v>1</v>
       </c>
-      <c r="K27" t="n">
+      <c r="N27" t="n">
         <v>3</v>
       </c>
-      <c r="L27" t="n">
-        <v>14</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0.7</v>
-      </c>
       <c r="O27" t="n">
-        <v>0.875</v>
+        <v>0.5806451612903226</v>
       </c>
       <c r="P27" t="n">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="R27" t="n">
-        <v>0.84</v>
+        <v>0.1</v>
       </c>
       <c r="S27" t="n">
-        <v>0.23</v>
+        <v>0.8</v>
       </c>
       <c r="T27" t="n">
-        <v>0.2533333333333333</v>
+        <v>0.48</v>
       </c>
       <c r="U27" t="n">
-        <v>0.2766666666666667</v>
+        <v>0.31</v>
+      </c>
+      <c r="V27" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.17</v>
       </c>
     </row>
     <row r="28">
@@ -2401,46 +2387,52 @@
         <v>0.2171606421470642</v>
       </c>
       <c r="H28" t="n">
+        <v>0.004134990740567446</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J28" t="n">
         <v>0.03543443605303764</v>
       </c>
-      <c r="I28" t="n">
-        <v>8</v>
-      </c>
-      <c r="J28" t="n">
-        <v>3</v>
-      </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L28" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M28" t="n">
-        <v>0.7619047619047619</v>
+        <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>0.8</v>
+        <v>5</v>
       </c>
       <c r="O28" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.6206896551724138</v>
       </c>
       <c r="P28" t="n">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.2</v>
+        <v>0.4736842105263158</v>
       </c>
       <c r="R28" t="n">
-        <v>0.8</v>
+        <v>0.1</v>
       </c>
       <c r="S28" t="n">
-        <v>0.2</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="T28" t="n">
-        <v>0.2</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="U28" t="n">
-        <v>0.2</v>
+        <v>0.27</v>
+      </c>
+      <c r="V28" t="n">
+        <v>0.2133333333333333</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.1566666666666667</v>
       </c>
     </row>
     <row r="29">
@@ -2463,55 +2455,61 @@
         <v>2012</v>
       </c>
       <c r="E29" t="n">
-        <v>0.8266666666666667</v>
+        <v>0.8266666666666668</v>
       </c>
       <c r="F29" t="n">
-        <v>0.8286247086247086</v>
+        <v>0.8184233158146201</v>
       </c>
       <c r="G29" t="n">
-        <v>0.1741227916710872</v>
+        <v>0.1738467908797114</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1691485916788619</v>
+        <v>0.1542737257044433</v>
       </c>
       <c r="I29" t="n">
-        <v>9</v>
+        <v>2011</v>
       </c>
       <c r="J29" t="n">
+        <v>0.1349760709410169</v>
+      </c>
+      <c r="K29" t="n">
+        <v>7</v>
+      </c>
+      <c r="L29" t="n">
         <v>4</v>
       </c>
-      <c r="K29" t="n">
-        <v>1</v>
-      </c>
-      <c r="L29" t="n">
+      <c r="M29" t="n">
+        <v>3</v>
+      </c>
+      <c r="N29" t="n">
         <v>11</v>
       </c>
-      <c r="M29" t="n">
-        <v>0.7826086956521739</v>
-      </c>
-      <c r="N29" t="n">
-        <v>0.9</v>
-      </c>
       <c r="O29" t="n">
-        <v>0.6923076923076923</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="P29" t="n">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="Q29" t="n">
+        <v>0.6363636363636364</v>
+      </c>
+      <c r="R29" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="S29" t="n">
         <v>0.2666666666666667</v>
       </c>
-      <c r="R29" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="S29" t="n">
-        <v>0.15</v>
-      </c>
       <c r="T29" t="n">
-        <v>0.1333333333333334</v>
+        <v>0.72</v>
       </c>
       <c r="U29" t="n">
-        <v>0.1166666666666667</v>
+        <v>0.29</v>
+      </c>
+      <c r="V29" t="n">
+        <v>0.2933333333333333</v>
+      </c>
+      <c r="W29" t="n">
+        <v>0.2966666666666667</v>
       </c>
     </row>
     <row r="30">
@@ -2534,54 +2532,60 @@
         <v>2012</v>
       </c>
       <c r="E30" t="n">
-        <v>0.5666666666666667</v>
+        <v>0.54</v>
       </c>
       <c r="F30" t="n">
         <v>0.4533333333333334</v>
       </c>
       <c r="G30" t="n">
-        <v>0.3511584918577925</v>
+        <v>0.3770100873979694</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
       </c>
       <c r="I30" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
         <v>10</v>
       </c>
-      <c r="J30" t="n">
+      <c r="L30" t="n">
         <v>15</v>
       </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
       <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
         <v>0.5714285714285714</v>
       </c>
-      <c r="N30" t="n">
+      <c r="P30" t="n">
         <v>1</v>
       </c>
-      <c r="O30" t="n">
+      <c r="Q30" t="n">
         <v>0.4</v>
       </c>
-      <c r="P30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" t="n">
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="n">
         <v>1</v>
       </c>
-      <c r="R30" t="n">
+      <c r="T30" t="n">
         <v>0.4</v>
       </c>
-      <c r="S30" t="n">
+      <c r="U30" t="n">
         <v>0.3</v>
       </c>
-      <c r="T30" t="n">
+      <c r="V30" t="n">
         <v>0.2</v>
       </c>
-      <c r="U30" t="n">
+      <c r="W30" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -2614,46 +2618,52 @@
         <v>0.2019680095014026</v>
       </c>
       <c r="H31" t="n">
+        <v>0.003988136469010892</v>
+      </c>
+      <c r="I31" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J31" t="n">
         <v>0.02090703665427157</v>
       </c>
-      <c r="I31" t="n">
+      <c r="K31" t="n">
         <v>9</v>
       </c>
-      <c r="J31" t="n">
-        <v>2</v>
-      </c>
-      <c r="K31" t="n">
+      <c r="L31" t="n">
+        <v>7</v>
+      </c>
+      <c r="M31" t="n">
         <v>1</v>
       </c>
-      <c r="L31" t="n">
-        <v>13</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0.8571428571428571</v>
-      </c>
       <c r="N31" t="n">
+        <v>8</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0.6923076923076923</v>
+      </c>
+      <c r="P31" t="n">
         <v>0.9</v>
       </c>
-      <c r="O31" t="n">
-        <v>0.8181818181818182</v>
-      </c>
-      <c r="P31" t="n">
+      <c r="Q31" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="R31" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q31" t="n">
-        <v>0.1333333333333333</v>
-      </c>
-      <c r="R31" t="n">
-        <v>0.88</v>
-      </c>
       <c r="S31" t="n">
-        <v>0.11</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="T31" t="n">
-        <v>0.1066666666666667</v>
+        <v>0.68</v>
       </c>
       <c r="U31" t="n">
-        <v>0.1033333333333333</v>
+        <v>0.21</v>
+      </c>
+      <c r="V31" t="n">
+        <v>0.1733333333333333</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0.1366666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -2689,7 +2699,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.603</v>
+        <v>0.583</v>
       </c>
     </row>
     <row r="3">
@@ -2699,7 +2709,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.782</v>
+        <v>0.756</v>
       </c>
     </row>
     <row r="4">
@@ -2709,7 +2719,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.638</v>
+        <v>0.636</v>
       </c>
     </row>
     <row r="5">
@@ -2719,7 +2729,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.627</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -2729,7 +2739,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.669</v>
       </c>
     </row>
     <row r="7">
@@ -2739,7 +2749,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.711</v>
+        <v>0.718</v>
       </c>
     </row>
   </sheetData>
@@ -2815,25 +2825,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.603</v>
+        <v>0.583</v>
       </c>
       <c r="D2" t="n">
-        <v>0.658</v>
+        <v>0.453</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="F2" t="n">
-        <v>0.533</v>
+        <v>0.375</v>
       </c>
       <c r="G2" t="n">
-        <v>0.067</v>
+        <v>0.3</v>
       </c>
       <c r="H2" t="n">
         <v>0.644</v>
       </c>
       <c r="I2" t="n">
-        <v>0.182</v>
+        <v>0.369</v>
       </c>
     </row>
     <row r="3">
@@ -2848,25 +2858,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.782</v>
+        <v>0.756</v>
       </c>
       <c r="D3" t="n">
-        <v>0.756</v>
+        <v>0.681</v>
       </c>
       <c r="E3" t="n">
-        <v>0.867</v>
+        <v>0.967</v>
       </c>
       <c r="F3" t="n">
-        <v>0.735</v>
+        <v>0.532</v>
       </c>
       <c r="G3" t="n">
-        <v>0.133</v>
+        <v>0.033</v>
       </c>
       <c r="H3" t="n">
-        <v>0.333</v>
+        <v>0.6</v>
       </c>
       <c r="I3" t="n">
-        <v>0.173</v>
+        <v>0.147</v>
       </c>
     </row>
     <row r="4">
@@ -2881,25 +2891,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.638</v>
+        <v>0.636</v>
       </c>
       <c r="D4" t="n">
-        <v>0.637</v>
+        <v>0.576</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="F4" t="n">
-        <v>0.505</v>
+        <v>0.463</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H4" t="n">
-        <v>0.644</v>
+        <v>0.667</v>
       </c>
       <c r="I4" t="n">
-        <v>0.209</v>
+        <v>0.293</v>
       </c>
     </row>
     <row r="5">
@@ -2914,25 +2924,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.627</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>0.648</v>
+        <v>0.541</v>
       </c>
       <c r="E5" t="n">
         <v>0.867</v>
       </c>
       <c r="F5" t="n">
-        <v>0.533</v>
+        <v>0.4</v>
       </c>
       <c r="G5" t="n">
         <v>0.133</v>
       </c>
       <c r="H5" t="n">
-        <v>0.556</v>
+        <v>0.867</v>
       </c>
       <c r="I5" t="n">
-        <v>0.218</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="6">
@@ -2947,25 +2957,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.669</v>
       </c>
       <c r="D6" t="n">
-        <v>0.721</v>
+        <v>0.666</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.967</v>
       </c>
       <c r="F6" t="n">
-        <v>0.645</v>
+        <v>0.523</v>
       </c>
       <c r="G6" t="n">
-        <v>0.067</v>
+        <v>0.033</v>
       </c>
       <c r="H6" t="n">
-        <v>0.511</v>
+        <v>0.667</v>
       </c>
       <c r="I6" t="n">
-        <v>0.156</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="7">
@@ -2980,25 +2990,25 @@
         </is>
       </c>
       <c r="C7" t="n">
+        <v>0.718</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.543</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.463</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H7" t="n">
         <v>0.711</v>
       </c>
-      <c r="D7" t="n">
-        <v>0.731</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.867</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.133</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.378</v>
-      </c>
       <c r="I7" t="n">
-        <v>0.182</v>
+        <v>0.302</v>
       </c>
     </row>
   </sheetData>
@@ -3044,7 +3054,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.603</v>
+        <v>0.583</v>
       </c>
     </row>
     <row r="3">
@@ -3054,7 +3064,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.782</v>
+        <v>0.756</v>
       </c>
     </row>
     <row r="4">
@@ -3064,7 +3074,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.638</v>
+        <v>0.636</v>
       </c>
     </row>
     <row r="5">
@@ -3074,7 +3084,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.627</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -3084,7 +3094,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.669</v>
       </c>
     </row>
     <row r="7">
@@ -3094,7 +3104,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.711</v>
+        <v>0.718</v>
       </c>
     </row>
     <row r="8">
@@ -3109,7 +3119,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.57</v>
+        <v>0.5570000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -3139,7 +3149,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.82</v>
+        <v>0.8169999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -3149,7 +3159,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.78</v>
+        <v>0.738</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Rerun the pre-crisis check on the corrected data (seed 99)
Same fixes as the seed 42 worktree: credit_gap_missing dropped at load in rt2b,
nfa_g replaced by nfa_gdp, 'crisis' excluded from micro_cols, threshold metrics
left empty (one test year has no evaluated predecessor), and the A46
falsification baseline added. rt2a/rt2b returned to tools/run_pipeline.py.

The falsification rule scores AUROC 1.000 here too.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/results/12a_gran/results_12a_isolate_gran_final.xlsx
+++ b/outputs/results/12a_gran/results_12a_isolate_gran_final.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:W31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,65 +462,75 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>threshold_from_year</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>test_optimal_threshold</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>tp</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>fp</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>fn</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>tn</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>f1</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>precision</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>miss_rate</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>false_alarm_rate</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>accuracy</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>loss_07</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>loss_08</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>loss_09</t>
         </is>
@@ -555,46 +565,52 @@
         <v>0.3302682062847694</v>
       </c>
       <c r="H2" t="n">
+        <v>0.4134512387890711</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J2" t="n">
         <v>0.01663706238879454</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L2" t="n">
         <v>10</v>
       </c>
-      <c r="J2" t="n">
-        <v>15</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
       <c r="M2" t="n">
-        <v>0.5714285714285714</v>
+        <v>4</v>
       </c>
       <c r="N2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O2" t="n">
-        <v>0.4</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>0.375</v>
       </c>
       <c r="R2" t="n">
         <v>0.4</v>
       </c>
       <c r="S2" t="n">
-        <v>0.3</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="T2" t="n">
-        <v>0.2</v>
+        <v>0.44</v>
       </c>
       <c r="U2" t="n">
-        <v>0.1</v>
+        <v>0.48</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.4533333333333334</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.4266666666666667</v>
       </c>
     </row>
     <row r="3">
@@ -617,55 +633,61 @@
         <v>2010</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5166666666666667</v>
+        <v>0.42</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4386503256468932</v>
+        <v>0.3551767676767676</v>
       </c>
       <c r="G3" t="n">
-        <v>0.247256</v>
+        <v>0.255936</v>
       </c>
       <c r="H3" t="n">
-        <v>0.32</v>
+        <v>0.03</v>
       </c>
       <c r="I3" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="K3" t="n">
         <v>10</v>
       </c>
-      <c r="J3" t="n">
-        <v>13</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
       <c r="L3" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6060606060606061</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" t="n">
-        <v>0.4347826086956522</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
       <c r="Q3" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.4</v>
       </c>
       <c r="R3" t="n">
-        <v>0.48</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0.26</v>
+        <v>1</v>
       </c>
       <c r="T3" t="n">
-        <v>0.1733333333333333</v>
+        <v>0.4</v>
       </c>
       <c r="U3" t="n">
-        <v>0.08666666666666667</v>
+        <v>0.3</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="4">
@@ -697,46 +719,52 @@
         <v>0.3515652120113373</v>
       </c>
       <c r="H4" t="n">
+        <v>0.01242134533822536</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J4" t="n">
         <v>0.3752442896366119</v>
       </c>
-      <c r="I4" t="n">
+      <c r="K4" t="n">
         <v>10</v>
       </c>
-      <c r="J4" t="n">
-        <v>12</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
       <c r="L4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="M4" t="n">
-        <v>0.625</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="n">
-        <v>0.4545454545454545</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
       <c r="Q4" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="R4" t="n">
-        <v>0.52</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>0.24</v>
+        <v>1</v>
       </c>
       <c r="T4" t="n">
-        <v>0.16</v>
+        <v>0.4</v>
       </c>
       <c r="U4" t="n">
-        <v>0.08000000000000002</v>
+        <v>0.3</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="5">
@@ -759,55 +787,61 @@
         <v>2010</v>
       </c>
       <c r="E5" t="n">
-        <v>0.44</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3808868908868909</v>
+        <v>0.405238167629472</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4000947300528722</v>
+        <v>0.395258511250831</v>
       </c>
       <c r="H5" t="n">
-        <v>0.03566289372715235</v>
+        <v>0.3138955698233886</v>
       </c>
       <c r="I5" t="n">
-        <v>10</v>
+        <v>2009</v>
       </c>
       <c r="J5" t="n">
-        <v>14</v>
+        <v>0.02073996970404562</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5882352941176471</v>
+        <v>4</v>
       </c>
       <c r="N5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="O5" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="R5" t="n">
-        <v>0.44</v>
+        <v>0.4</v>
       </c>
       <c r="S5" t="n">
-        <v>0.28</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="T5" t="n">
-        <v>0.1866666666666667</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="U5" t="n">
-        <v>0.09333333333333334</v>
+        <v>0.4199999999999999</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.4133333333333334</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.4066666666666667</v>
       </c>
     </row>
     <row r="6">
@@ -830,55 +864,61 @@
         <v>2010</v>
       </c>
       <c r="E6" t="n">
-        <v>0.45</v>
+        <v>0.42</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3988636363636364</v>
+        <v>0.3954545454545455</v>
       </c>
       <c r="G6" t="n">
-        <v>0.379083972587156</v>
+        <v>0.3825089562866688</v>
       </c>
       <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J6" t="n">
         <v>0.420814479638009</v>
       </c>
-      <c r="I6" t="n">
+      <c r="K6" t="n">
         <v>10</v>
       </c>
-      <c r="J6" t="n">
-        <v>14</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
       <c r="L6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P6" t="n">
         <v>1</v>
       </c>
-      <c r="M6" t="n">
-        <v>0.5882352941176471</v>
-      </c>
-      <c r="N6" t="n">
+      <c r="Q6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
         <v>1</v>
       </c>
-      <c r="O6" t="n">
-        <v>0.4166666666666667</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.9333333333333333</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.28</v>
-      </c>
       <c r="T6" t="n">
-        <v>0.1866666666666667</v>
+        <v>0.4</v>
       </c>
       <c r="U6" t="n">
-        <v>0.09333333333333334</v>
+        <v>0.3</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="7">
@@ -910,45 +950,51 @@
         <v>0.3083624220446608</v>
       </c>
       <c r="H7" t="n">
+        <v>0.04470937183400933</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2009</v>
+      </c>
+      <c r="J7" t="n">
         <v>0.1188634608818508</v>
       </c>
-      <c r="I7" t="n">
+      <c r="K7" t="n">
         <v>10</v>
       </c>
-      <c r="J7" t="n">
+      <c r="L7" t="n">
         <v>12</v>
       </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
         <v>3</v>
       </c>
-      <c r="M7" t="n">
+      <c r="O7" t="n">
         <v>0.625</v>
       </c>
-      <c r="N7" t="n">
+      <c r="P7" t="n">
         <v>1</v>
       </c>
-      <c r="O7" t="n">
+      <c r="Q7" t="n">
         <v>0.4545454545454545</v>
       </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
         <v>0.8</v>
       </c>
-      <c r="R7" t="n">
+      <c r="T7" t="n">
         <v>0.52</v>
       </c>
-      <c r="S7" t="n">
+      <c r="U7" t="n">
         <v>0.24</v>
       </c>
-      <c r="T7" t="n">
+      <c r="V7" t="n">
         <v>0.16</v>
       </c>
-      <c r="U7" t="n">
+      <c r="W7" t="n">
         <v>0.08000000000000002</v>
       </c>
     </row>
@@ -972,55 +1018,61 @@
         <v>2011</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.66</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6510926399545325</v>
+        <v>0.6472464861083786</v>
       </c>
       <c r="G8" t="n">
-        <v>0.24142315899945</v>
+        <v>0.242335169490867</v>
       </c>
       <c r="H8" t="n">
-        <v>0.479564160817484</v>
+        <v>0.01663706238879454</v>
       </c>
       <c r="I8" t="n">
-        <v>9</v>
+        <v>2010</v>
       </c>
       <c r="J8" t="n">
-        <v>9</v>
+        <v>0.482023971522149</v>
       </c>
       <c r="K8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" t="n">
+        <v>15</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="P8" t="n">
         <v>1</v>
       </c>
-      <c r="L8" t="n">
-        <v>6</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.6428571428571429</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W8" t="n">
         <v>0.1</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="U8" t="n">
-        <v>0.15</v>
       </c>
     </row>
     <row r="9">
@@ -1043,55 +1095,61 @@
         <v>2011</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6533333333333333</v>
+        <v>0.6733333333333333</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5856434793276898</v>
+        <v>0.6080237358101134</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2230026896503645</v>
+        <v>0.2237022748530627</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3845475210954841</v>
+        <v>0.34</v>
       </c>
       <c r="I9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.3972538540055997</v>
+      </c>
+      <c r="K9" t="n">
         <v>10</v>
       </c>
-      <c r="J9" t="n">
-        <v>10</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
       <c r="L9" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="M9" t="n">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="P9" t="n">
         <v>1</v>
       </c>
-      <c r="O9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
       <c r="Q9" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4545454545454545</v>
       </c>
       <c r="R9" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="T9" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.52</v>
       </c>
       <c r="U9" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.24</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.08000000000000002</v>
       </c>
     </row>
     <row r="10">
@@ -1114,55 +1172,61 @@
         <v>2011</v>
       </c>
       <c r="E10" t="n">
-        <v>0.7533333333333334</v>
+        <v>0.7666666666666667</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6665909090909091</v>
+        <v>0.6814729225023343</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2561646401882172</v>
+        <v>0.2635264098644257</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1051026284694672</v>
+        <v>0.3752442896366119</v>
       </c>
       <c r="I10" t="n">
-        <v>8</v>
+        <v>2010</v>
       </c>
       <c r="J10" t="n">
-        <v>4</v>
+        <v>0.1295015811920166</v>
       </c>
       <c r="K10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L10" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
-        <v>0.7272727272727273</v>
+        <v>7</v>
       </c>
       <c r="N10" t="n">
-        <v>0.8</v>
+        <v>12</v>
       </c>
       <c r="O10" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.375</v>
       </c>
       <c r="P10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="S10" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q10" t="n">
-        <v>0.2666666666666667</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0.22</v>
-      </c>
       <c r="T10" t="n">
-        <v>0.2133333333333334</v>
+        <v>0.6</v>
       </c>
       <c r="U10" t="n">
-        <v>0.2066666666666667</v>
+        <v>0.5499999999999999</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.65</v>
       </c>
     </row>
     <row r="11">
@@ -1185,55 +1249,61 @@
         <v>2011</v>
       </c>
       <c r="E11" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="F11" t="n">
-        <v>0.6983467023172906</v>
+        <v>0.691220397249809</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2332489029133263</v>
+        <v>0.2318080346328482</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4910117331747179</v>
+        <v>0.02073996970404562</v>
       </c>
       <c r="I11" t="n">
-        <v>7</v>
+        <v>2010</v>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>0.478869509698488</v>
       </c>
       <c r="K11" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="M11" t="n">
-        <v>0.6363636363636364</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="P11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U11" t="n">
         <v>0.3</v>
       </c>
-      <c r="Q11" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="T11" t="n">
-        <v>0.3066666666666666</v>
-      </c>
-      <c r="U11" t="n">
-        <v>0.3033333333333333</v>
+      <c r="V11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="12">
@@ -1256,55 +1326,61 @@
         <v>2011</v>
       </c>
       <c r="E12" t="n">
-        <v>0.5366666666666666</v>
+        <v>0.5066666666666666</v>
       </c>
       <c r="F12" t="n">
-        <v>0.4340909090909091</v>
+        <v>0.42</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2656166240652603</v>
+        <v>0.3830235750004732</v>
       </c>
       <c r="H12" t="n">
-        <v>0.3287671232876714</v>
+        <v>0.420814479638009</v>
       </c>
       <c r="I12" t="n">
-        <v>10</v>
+        <v>2010</v>
       </c>
       <c r="J12" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L12" t="n">
         <v>3</v>
       </c>
       <c r="M12" t="n">
-        <v>0.625</v>
+        <v>8</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="O12" t="n">
-        <v>0.4545454545454545</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="Q12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R12" t="n">
         <v>0.8</v>
       </c>
-      <c r="R12" t="n">
-        <v>0.52</v>
-      </c>
       <c r="S12" t="n">
-        <v>0.24</v>
+        <v>0.2</v>
       </c>
       <c r="T12" t="n">
-        <v>0.16</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="U12" t="n">
-        <v>0.08000000000000002</v>
+        <v>0.6199999999999999</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.6800000000000002</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.7400000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -1327,55 +1403,61 @@
         <v>2011</v>
       </c>
       <c r="E13" t="n">
-        <v>0.88</v>
+        <v>0.7733333333333334</v>
       </c>
       <c r="F13" t="n">
-        <v>0.8263383838383839</v>
+        <v>0.668015873015873</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2879982548758644</v>
+        <v>0.2323889794490995</v>
       </c>
       <c r="H13" t="n">
-        <v>0.005595969106936115</v>
+        <v>0.1188634608818508</v>
       </c>
       <c r="I13" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.2411839014309663</v>
+      </c>
+      <c r="K13" t="n">
+        <v>7</v>
+      </c>
+      <c r="L13" t="n">
+        <v>6</v>
+      </c>
+      <c r="M13" t="n">
+        <v>3</v>
+      </c>
+      <c r="N13" t="n">
         <v>9</v>
       </c>
-      <c r="J13" t="n">
-        <v>3</v>
-      </c>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13" t="n">
-        <v>12</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.8181818181818182</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0.9</v>
-      </c>
       <c r="O13" t="n">
-        <v>0.75</v>
+        <v>0.6086956521739131</v>
       </c>
       <c r="P13" t="n">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.2</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="R13" t="n">
-        <v>0.84</v>
+        <v>0.3</v>
       </c>
       <c r="S13" t="n">
-        <v>0.13</v>
+        <v>0.4</v>
       </c>
       <c r="T13" t="n">
-        <v>0.12</v>
+        <v>0.64</v>
       </c>
       <c r="U13" t="n">
-        <v>0.11</v>
+        <v>0.33</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.3100000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -1404,49 +1486,55 @@
         <v>0.7106672494172493</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2015931568180839</v>
+        <v>0.2020669989268483</v>
       </c>
       <c r="H14" t="n">
-        <v>0.4839371869283402</v>
+        <v>0.482023971522149</v>
       </c>
       <c r="I14" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.4833176805530612</v>
+      </c>
+      <c r="K14" t="n">
         <v>8</v>
       </c>
-      <c r="J14" t="n">
-        <v>5</v>
-      </c>
-      <c r="K14" t="n">
+      <c r="L14" t="n">
+        <v>6</v>
+      </c>
+      <c r="M14" t="n">
         <v>2</v>
       </c>
-      <c r="L14" t="n">
-        <v>10</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0.6956521739130435</v>
-      </c>
       <c r="N14" t="n">
+        <v>9</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="P14" t="n">
         <v>0.8</v>
       </c>
-      <c r="O14" t="n">
-        <v>0.6153846153846154</v>
-      </c>
-      <c r="P14" t="n">
+      <c r="Q14" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="R14" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q14" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0.72</v>
-      </c>
       <c r="S14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="V14" t="n">
         <v>0.24</v>
       </c>
-      <c r="T14" t="n">
-        <v>0.2266666666666667</v>
-      </c>
-      <c r="U14" t="n">
-        <v>0.2133333333333333</v>
+      <c r="W14" t="n">
+        <v>0.22</v>
       </c>
     </row>
     <row r="15">
@@ -1469,55 +1557,61 @@
         <v>2012</v>
       </c>
       <c r="E15" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.9500000000000001</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.1364285714285714</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.3972538540055997</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.4464285714285715</v>
+      </c>
+      <c r="K15" t="n">
+        <v>9</v>
+      </c>
+      <c r="L15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="n">
+        <v>12</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="P15" t="n">
         <v>0.9</v>
       </c>
-      <c r="F15" t="n">
-        <v>0.9126315789473685</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.1729535948149485</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.6117757361783286</v>
-      </c>
-      <c r="I15" t="n">
-        <v>8</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>2</v>
-      </c>
-      <c r="L15" t="n">
-        <v>15</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O15" t="n">
-        <v>1</v>
-      </c>
-      <c r="P15" t="n">
+      <c r="Q15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S15" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="S15" t="n">
-        <v>0.14</v>
-      </c>
       <c r="T15" t="n">
-        <v>0.16</v>
+        <v>0.84</v>
       </c>
       <c r="U15" t="n">
-        <v>0.18</v>
+        <v>0.13</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0.11</v>
       </c>
     </row>
     <row r="16">
@@ -1540,55 +1634,61 @@
         <v>2012</v>
       </c>
       <c r="E16" t="n">
-        <v>0.8733333333333334</v>
+        <v>0.7933333333333333</v>
       </c>
       <c r="F16" t="n">
-        <v>0.8826388888888889</v>
+        <v>0.7948051948051947</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1501580774784088</v>
+        <v>0.1985791921615601</v>
       </c>
       <c r="H16" t="n">
-        <v>0.671759307384491</v>
+        <v>0.1295015811920166</v>
       </c>
       <c r="I16" t="n">
-        <v>8</v>
+        <v>2011</v>
       </c>
       <c r="J16" t="n">
+        <v>0.5760293006896973</v>
+      </c>
+      <c r="K16" t="n">
+        <v>9</v>
+      </c>
+      <c r="L16" t="n">
+        <v>9</v>
+      </c>
+      <c r="M16" t="n">
         <v>1</v>
       </c>
-      <c r="K16" t="n">
-        <v>2</v>
-      </c>
-      <c r="L16" t="n">
-        <v>14</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0.8421052631578947</v>
-      </c>
       <c r="N16" t="n">
-        <v>0.8</v>
+        <v>6</v>
       </c>
       <c r="O16" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="P16" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="T16" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="V16" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q16" t="n">
-        <v>0.06666666666666667</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="S16" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="T16" t="n">
-        <v>0.1733333333333334</v>
-      </c>
-      <c r="U16" t="n">
-        <v>0.1866666666666667</v>
+      <c r="W16" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="17">
@@ -1611,55 +1711,61 @@
         <v>2012</v>
       </c>
       <c r="E17" t="n">
-        <v>0.74</v>
+        <v>0.7266666666666667</v>
       </c>
       <c r="F17" t="n">
-        <v>0.7488677988677989</v>
+        <v>0.7034920634920635</v>
       </c>
       <c r="G17" t="n">
-        <v>0.217466614056738</v>
+        <v>0.2824134255195166</v>
       </c>
       <c r="H17" t="n">
-        <v>0.4996605725769222</v>
+        <v>0.478869509698488</v>
       </c>
       <c r="I17" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.6615682750040593</v>
+      </c>
+      <c r="K17" t="n">
         <v>9</v>
       </c>
-      <c r="J17" t="n">
-        <v>6</v>
-      </c>
-      <c r="K17" t="n">
+      <c r="L17" t="n">
+        <v>15</v>
+      </c>
+      <c r="M17" t="n">
         <v>1</v>
       </c>
-      <c r="L17" t="n">
-        <v>9</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0.72</v>
-      </c>
       <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.5294117647058824</v>
+      </c>
+      <c r="P17" t="n">
         <v>0.9</v>
       </c>
-      <c r="O17" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="P17" t="n">
+      <c r="Q17" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="R17" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q17" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="R17" t="n">
-        <v>0.72</v>
-      </c>
       <c r="S17" t="n">
+        <v>1</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="W17" t="n">
         <v>0.19</v>
-      </c>
-      <c r="T17" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U17" t="n">
-        <v>0.13</v>
       </c>
     </row>
     <row r="18">
@@ -1682,55 +1788,61 @@
         <v>2012</v>
       </c>
       <c r="E18" t="n">
-        <v>0.8233333333333334</v>
+        <v>0.7333333333333334</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7257575757575758</v>
+        <v>0.61</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1841320532431732</v>
+        <v>0.24</v>
       </c>
       <c r="H18" t="n">
-        <v>0.7374566109182709</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>8</v>
+        <v>2011</v>
       </c>
       <c r="J18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L18" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M18" t="n">
-        <v>0.7619047619047619</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="P18" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V18" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q18" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="R18" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="S18" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="T18" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="U18" t="n">
-        <v>0.2</v>
+      <c r="W18" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="19">
@@ -1753,55 +1865,61 @@
         <v>2012</v>
       </c>
       <c r="E19" t="n">
+        <v>0.9266666666666667</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.9344497607655503</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.1075111221063298</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.2411839014309663</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.6446247244195131</v>
+      </c>
+      <c r="K19" t="n">
+        <v>9</v>
+      </c>
+      <c r="L19" t="n">
+        <v>6</v>
+      </c>
+      <c r="M19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" t="n">
+        <v>9</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="P19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F19" t="n">
-        <v>0.9003588516746411</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.1384474904804223</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0.7285815117256835</v>
-      </c>
-      <c r="I19" t="n">
-        <v>7</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L19" t="n">
-        <v>15</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0.8235294117647058</v>
-      </c>
-      <c r="N19" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="O19" t="n">
-        <v>1</v>
-      </c>
-      <c r="P19" t="n">
-        <v>0.3</v>
-      </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="R19" t="n">
-        <v>0.88</v>
+        <v>0.1</v>
       </c>
       <c r="S19" t="n">
-        <v>0.21</v>
+        <v>0.4</v>
       </c>
       <c r="T19" t="n">
-        <v>0.24</v>
+        <v>0.72</v>
       </c>
       <c r="U19" t="n">
-        <v>0.27</v>
+        <v>0.19</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.13</v>
       </c>
     </row>
     <row r="20">
@@ -1832,48 +1950,24 @@
       <c r="G20" t="n">
         <v>0.2155429920581876</v>
       </c>
-      <c r="H20" t="n">
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="n">
         <v>0.214396107376168</v>
       </c>
-      <c r="I20" t="n">
-        <v>8</v>
-      </c>
-      <c r="J20" t="n">
-        <v>6</v>
-      </c>
-      <c r="K20" t="n">
-        <v>2</v>
-      </c>
-      <c r="L20" t="n">
-        <v>9</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="S20" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="T20" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="U20" t="n">
-        <v>0.22</v>
-      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1895,56 +1989,32 @@
         <v>2011</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6733333333333333</v>
+        <v>0.6433333333333333</v>
       </c>
       <c r="F21" t="n">
-        <v>0.6533760683760683</v>
+        <v>0.6156782106782106</v>
       </c>
       <c r="G21" t="n">
-        <v>0.3209719999999999</v>
-      </c>
-      <c r="H21" t="n">
+        <v>0.326176</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="n">
         <v>0.02</v>
       </c>
-      <c r="I21" t="n">
-        <v>8</v>
-      </c>
-      <c r="J21" t="n">
-        <v>8</v>
-      </c>
-      <c r="K21" t="n">
-        <v>2</v>
-      </c>
-      <c r="L21" t="n">
-        <v>7</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.6153846153846154</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0.5333333333333333</v>
-      </c>
-      <c r="R21" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="S21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T21" t="n">
-        <v>0.2666666666666667</v>
-      </c>
-      <c r="U21" t="n">
-        <v>0.2333333333333334</v>
-      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1974,48 +2044,24 @@
       <c r="G22" t="n">
         <v>0.312720388174057</v>
       </c>
-      <c r="H22" t="n">
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="n">
         <v>0.004134990740567446</v>
       </c>
-      <c r="I22" t="n">
-        <v>9</v>
-      </c>
-      <c r="J22" t="n">
-        <v>8</v>
-      </c>
-      <c r="K22" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" t="n">
-        <v>7</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0.5294117647058824</v>
-      </c>
-      <c r="P22" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>0.5333333333333333</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="S22" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="T22" t="n">
-        <v>0.1866666666666667</v>
-      </c>
-      <c r="U22" t="n">
-        <v>0.1433333333333333</v>
-      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2037,56 +2083,32 @@
         <v>2011</v>
       </c>
       <c r="E23" t="n">
-        <v>0.8133333333333334</v>
+        <v>0.84</v>
       </c>
       <c r="F23" t="n">
-        <v>0.798799762329174</v>
+        <v>0.8127231020613374</v>
       </c>
       <c r="G23" t="n">
-        <v>0.1911382389981019</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.1807592812230448</v>
-      </c>
-      <c r="I23" t="n">
-        <v>8</v>
-      </c>
+        <v>0.1751446582528155</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="n">
-        <v>4</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>11</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0.7272727272727273</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="P23" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>0.2666666666666667</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="S23" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="T23" t="n">
-        <v>0.2133333333333334</v>
-      </c>
-      <c r="U23" t="n">
-        <v>0.2066666666666667</v>
-      </c>
+        <v>0.1225095633950481</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2116,48 +2138,24 @@
       <c r="G24" t="n">
         <v>0.3427203439871637</v>
       </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>10</v>
-      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="n">
-        <v>15</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="N24" t="n">
-        <v>1</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1</v>
-      </c>
-      <c r="R24" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S24" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T24" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="U24" t="n">
-        <v>0.1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2187,48 +2185,24 @@
       <c r="G25" t="n">
         <v>0.2764459795613017</v>
       </c>
-      <c r="H25" t="n">
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="n">
         <v>0.003988136469010892</v>
       </c>
-      <c r="I25" t="n">
-        <v>8</v>
-      </c>
-      <c r="J25" t="n">
-        <v>1</v>
-      </c>
-      <c r="K25" t="n">
-        <v>2</v>
-      </c>
-      <c r="L25" t="n">
-        <v>14</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0.8421052631578947</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="P25" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>0.06666666666666667</v>
-      </c>
-      <c r="R25" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="S25" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="T25" t="n">
-        <v>0.1733333333333334</v>
-      </c>
-      <c r="U25" t="n">
-        <v>0.1866666666666667</v>
-      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2259,46 +2233,52 @@
         <v>0.1831261321893823</v>
       </c>
       <c r="H26" t="n">
+        <v>0.214396107376168</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J26" t="n">
         <v>0.1466912697483659</v>
       </c>
-      <c r="I26" t="n">
-        <v>10</v>
-      </c>
-      <c r="J26" t="n">
-        <v>7</v>
-      </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L26" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M26" t="n">
-        <v>0.7407407407407407</v>
+        <v>4</v>
       </c>
       <c r="N26" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="O26" t="n">
-        <v>0.5882352941176471</v>
+        <v>0.6</v>
       </c>
       <c r="P26" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.4666666666666667</v>
+        <v>0.6</v>
       </c>
       <c r="R26" t="n">
-        <v>0.72</v>
+        <v>0.4</v>
       </c>
       <c r="S26" t="n">
-        <v>0.14</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="T26" t="n">
-        <v>0.09333333333333334</v>
+        <v>0.68</v>
       </c>
       <c r="U26" t="n">
-        <v>0.04666666666666667</v>
+        <v>0.36</v>
+      </c>
+      <c r="V26" t="n">
+        <v>0.3733333333333334</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.3866666666666667</v>
       </c>
     </row>
     <row r="27">
@@ -2324,52 +2304,58 @@
         <v>0.8866666666666666</v>
       </c>
       <c r="F27" t="n">
-        <v>0.8323841354723708</v>
+        <v>0.8793055555555555</v>
       </c>
       <c r="G27" t="n">
-        <v>0.216776</v>
+        <v>0.218724</v>
       </c>
       <c r="H27" t="n">
-        <v>0.25</v>
+        <v>0.02</v>
       </c>
       <c r="I27" t="n">
-        <v>7</v>
+        <v>2011</v>
       </c>
       <c r="J27" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="K27" t="n">
+        <v>10</v>
+      </c>
+      <c r="L27" t="n">
+        <v>12</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>3</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="P27" t="n">
         <v>1</v>
       </c>
-      <c r="K27" t="n">
-        <v>3</v>
-      </c>
-      <c r="L27" t="n">
-        <v>14</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="O27" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="P27" t="n">
-        <v>0.3</v>
-      </c>
       <c r="Q27" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.4545454545454545</v>
       </c>
       <c r="R27" t="n">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>0.23</v>
+        <v>0.8</v>
       </c>
       <c r="T27" t="n">
-        <v>0.2533333333333333</v>
+        <v>0.52</v>
       </c>
       <c r="U27" t="n">
-        <v>0.2766666666666667</v>
+        <v>0.24</v>
+      </c>
+      <c r="V27" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.08000000000000002</v>
       </c>
     </row>
     <row r="28">
@@ -2401,46 +2387,52 @@
         <v>0.2171606421470642</v>
       </c>
       <c r="H28" t="n">
+        <v>0.004134990740567446</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J28" t="n">
         <v>0.03543443605303764</v>
       </c>
-      <c r="I28" t="n">
-        <v>8</v>
-      </c>
-      <c r="J28" t="n">
-        <v>3</v>
-      </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L28" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M28" t="n">
-        <v>0.7619047619047619</v>
+        <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>0.8</v>
+        <v>5</v>
       </c>
       <c r="O28" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.6206896551724138</v>
       </c>
       <c r="P28" t="n">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.2</v>
+        <v>0.4736842105263158</v>
       </c>
       <c r="R28" t="n">
-        <v>0.8</v>
+        <v>0.1</v>
       </c>
       <c r="S28" t="n">
-        <v>0.2</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="T28" t="n">
-        <v>0.2</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="U28" t="n">
-        <v>0.2</v>
+        <v>0.27</v>
+      </c>
+      <c r="V28" t="n">
+        <v>0.2133333333333333</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.1566666666666667</v>
       </c>
     </row>
     <row r="29">
@@ -2463,54 +2455,60 @@
         <v>2012</v>
       </c>
       <c r="E29" t="n">
-        <v>0.8266666666666667</v>
+        <v>0.8200000000000001</v>
       </c>
       <c r="F29" t="n">
-        <v>0.8286247086247086</v>
+        <v>0.7668498168498168</v>
       </c>
       <c r="G29" t="n">
-        <v>0.1741227916710872</v>
+        <v>0.1835174498836435</v>
       </c>
       <c r="H29" t="n">
-        <v>0.1691485916788619</v>
+        <v>0.1225095633950481</v>
       </c>
       <c r="I29" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.1504589925383826</v>
+      </c>
+      <c r="K29" t="n">
         <v>9</v>
       </c>
-      <c r="J29" t="n">
+      <c r="L29" t="n">
         <v>4</v>
       </c>
-      <c r="K29" t="n">
+      <c r="M29" t="n">
         <v>1</v>
       </c>
-      <c r="L29" t="n">
+      <c r="N29" t="n">
         <v>11</v>
       </c>
-      <c r="M29" t="n">
+      <c r="O29" t="n">
         <v>0.7826086956521739</v>
       </c>
-      <c r="N29" t="n">
+      <c r="P29" t="n">
         <v>0.9</v>
       </c>
-      <c r="O29" t="n">
+      <c r="Q29" t="n">
         <v>0.6923076923076923</v>
       </c>
-      <c r="P29" t="n">
+      <c r="R29" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q29" t="n">
+      <c r="S29" t="n">
         <v>0.2666666666666667</v>
       </c>
-      <c r="R29" t="n">
+      <c r="T29" t="n">
         <v>0.8</v>
       </c>
-      <c r="S29" t="n">
+      <c r="U29" t="n">
         <v>0.15</v>
       </c>
-      <c r="T29" t="n">
+      <c r="V29" t="n">
         <v>0.1333333333333334</v>
       </c>
-      <c r="U29" t="n">
+      <c r="W29" t="n">
         <v>0.1166666666666667</v>
       </c>
     </row>
@@ -2546,42 +2544,48 @@
         <v>0</v>
       </c>
       <c r="I30" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
         <v>10</v>
       </c>
-      <c r="J30" t="n">
+      <c r="L30" t="n">
         <v>15</v>
       </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
       <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
         <v>0.5714285714285714</v>
       </c>
-      <c r="N30" t="n">
+      <c r="P30" t="n">
         <v>1</v>
       </c>
-      <c r="O30" t="n">
+      <c r="Q30" t="n">
         <v>0.4</v>
       </c>
-      <c r="P30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" t="n">
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="n">
         <v>1</v>
       </c>
-      <c r="R30" t="n">
+      <c r="T30" t="n">
         <v>0.4</v>
       </c>
-      <c r="S30" t="n">
+      <c r="U30" t="n">
         <v>0.3</v>
       </c>
-      <c r="T30" t="n">
+      <c r="V30" t="n">
         <v>0.2</v>
       </c>
-      <c r="U30" t="n">
+      <c r="W30" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -2614,46 +2618,52 @@
         <v>0.2019680095014026</v>
       </c>
       <c r="H31" t="n">
+        <v>0.003988136469010892</v>
+      </c>
+      <c r="I31" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J31" t="n">
         <v>0.02090703665427157</v>
       </c>
-      <c r="I31" t="n">
+      <c r="K31" t="n">
         <v>9</v>
       </c>
-      <c r="J31" t="n">
-        <v>2</v>
-      </c>
-      <c r="K31" t="n">
+      <c r="L31" t="n">
+        <v>7</v>
+      </c>
+      <c r="M31" t="n">
         <v>1</v>
       </c>
-      <c r="L31" t="n">
-        <v>13</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0.8571428571428571</v>
-      </c>
       <c r="N31" t="n">
+        <v>8</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0.6923076923076923</v>
+      </c>
+      <c r="P31" t="n">
         <v>0.9</v>
       </c>
-      <c r="O31" t="n">
-        <v>0.8181818181818182</v>
-      </c>
-      <c r="P31" t="n">
+      <c r="Q31" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="R31" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q31" t="n">
-        <v>0.1333333333333333</v>
-      </c>
-      <c r="R31" t="n">
-        <v>0.88</v>
-      </c>
       <c r="S31" t="n">
-        <v>0.11</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="T31" t="n">
-        <v>0.1066666666666667</v>
+        <v>0.68</v>
       </c>
       <c r="U31" t="n">
-        <v>0.1033333333333333</v>
+        <v>0.21</v>
+      </c>
+      <c r="V31" t="n">
+        <v>0.1733333333333333</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0.1366666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -2689,7 +2699,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.603</v>
+        <v>0.553</v>
       </c>
     </row>
     <row r="3">
@@ -2699,7 +2709,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.782</v>
+        <v>0.756</v>
       </c>
     </row>
     <row r="4">
@@ -2709,7 +2719,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.638</v>
+        <v>0.636</v>
       </c>
     </row>
     <row r="5">
@@ -2719,7 +2729,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.627</v>
+        <v>0.638</v>
       </c>
     </row>
     <row r="6">
@@ -2729,7 +2739,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.676</v>
       </c>
     </row>
     <row r="7">
@@ -2739,7 +2749,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.711</v>
+        <v>0.6889999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2815,25 +2825,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.603</v>
+        <v>0.553</v>
       </c>
       <c r="D2" t="n">
-        <v>0.658</v>
+        <v>0.47</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.733</v>
       </c>
       <c r="F2" t="n">
-        <v>0.533</v>
+        <v>0.4</v>
       </c>
       <c r="G2" t="n">
-        <v>0.067</v>
+        <v>0.267</v>
       </c>
       <c r="H2" t="n">
-        <v>0.644</v>
+        <v>0.733</v>
       </c>
       <c r="I2" t="n">
-        <v>0.182</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="3">
@@ -2848,25 +2858,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.782</v>
+        <v>0.756</v>
       </c>
       <c r="D3" t="n">
-        <v>0.756</v>
+        <v>0.651</v>
       </c>
       <c r="E3" t="n">
         <v>0.867</v>
       </c>
       <c r="F3" t="n">
-        <v>0.735</v>
+        <v>0.531</v>
       </c>
       <c r="G3" t="n">
         <v>0.133</v>
       </c>
       <c r="H3" t="n">
-        <v>0.333</v>
+        <v>0.533</v>
       </c>
       <c r="I3" t="n">
-        <v>0.173</v>
+        <v>0.213</v>
       </c>
     </row>
     <row r="4">
@@ -2881,25 +2891,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.638</v>
+        <v>0.636</v>
       </c>
       <c r="D4" t="n">
-        <v>0.637</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="F4" t="n">
-        <v>0.505</v>
+        <v>0.449</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H4" t="n">
-        <v>0.644</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>0.209</v>
+        <v>0.298</v>
       </c>
     </row>
     <row r="5">
@@ -2914,25 +2924,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.627</v>
+        <v>0.638</v>
       </c>
       <c r="D5" t="n">
-        <v>0.648</v>
+        <v>0.541</v>
       </c>
       <c r="E5" t="n">
-        <v>0.867</v>
+        <v>0.833</v>
       </c>
       <c r="F5" t="n">
-        <v>0.533</v>
+        <v>0.412</v>
       </c>
       <c r="G5" t="n">
-        <v>0.133</v>
+        <v>0.167</v>
       </c>
       <c r="H5" t="n">
-        <v>0.556</v>
+        <v>0.822</v>
       </c>
       <c r="I5" t="n">
-        <v>0.218</v>
+        <v>0.298</v>
       </c>
     </row>
     <row r="6">
@@ -2947,25 +2957,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.676</v>
       </c>
       <c r="D6" t="n">
-        <v>0.721</v>
+        <v>0.672</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.967</v>
       </c>
       <c r="F6" t="n">
-        <v>0.645</v>
+        <v>0.535</v>
       </c>
       <c r="G6" t="n">
-        <v>0.067</v>
+        <v>0.033</v>
       </c>
       <c r="H6" t="n">
-        <v>0.511</v>
+        <v>0.667</v>
       </c>
       <c r="I6" t="n">
-        <v>0.156</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="7">
@@ -2980,25 +2990,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.711</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>0.731</v>
+        <v>0.53</v>
       </c>
       <c r="E7" t="n">
-        <v>0.867</v>
+        <v>0.733</v>
       </c>
       <c r="F7" t="n">
-        <v>0.67</v>
+        <v>0.467</v>
       </c>
       <c r="G7" t="n">
-        <v>0.133</v>
+        <v>0.267</v>
       </c>
       <c r="H7" t="n">
-        <v>0.378</v>
+        <v>0.6</v>
       </c>
       <c r="I7" t="n">
-        <v>0.182</v>
+        <v>0.333</v>
       </c>
     </row>
   </sheetData>
@@ -3044,7 +3054,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.603</v>
+        <v>0.553</v>
       </c>
     </row>
     <row r="3">
@@ -3054,7 +3064,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.782</v>
+        <v>0.756</v>
       </c>
     </row>
     <row r="4">
@@ -3064,7 +3074,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.638</v>
+        <v>0.636</v>
       </c>
     </row>
     <row r="5">
@@ -3074,7 +3084,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.627</v>
+        <v>0.638</v>
       </c>
     </row>
     <row r="6">
@@ -3084,7 +3094,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.676</v>
       </c>
     </row>
     <row r="7">
@@ -3094,7 +3104,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.711</v>
+        <v>0.6889999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -3139,7 +3149,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="12">
@@ -3149,7 +3159,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.78</v>
+        <v>0.765</v>
       </c>
     </row>
     <row r="13">

</xml_diff>